<commit_message>
Recompile Fortran engines using Visual Studio 2026 and Intel® Fortran Compiler 2026.0.0.
</commit_message>
<xml_diff>
--- a/RegexFeatureMatrix.xlsx
+++ b/RegexFeatureMatrix.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="R79e52b8b2bc34ea0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="R9e87c771b89d48a5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -91,7 +91,7 @@
   </x:si>
   <x:si>
     <x:t>Fortran (IFX)
- 2025.3.0 </x:t>
+ 2026.0.0 </x:t>
   </x:si>
   <x:si>
     <x:t>TRE
@@ -1000,7 +1000,7 @@
     <x:t>(?P=name)</x:t>
   </x:si>
   <x:si>
-    <x:t>Grouping</x:t>
+    <x:t>Grouping and Lookaround</x:t>
   </x:si>
   <x:si>
     <x:t>(?:…)</x:t>

</xml_diff>

<commit_message>
Update RE2JS engine: 2.8.3.
</commit_message>
<xml_diff>
--- a/RegexFeatureMatrix.xlsx
+++ b/RegexFeatureMatrix.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="Rde96327c53be477b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="Rd7de7708dc794e7f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1265,7 +1265,7 @@
     <x:t>Approximate matching using special patterns or parameters</x:t>
   </x:si>
   <x:si>
-    <x:t>No hang</x:t>
+    <x:t>No hang, no ReDoS</x:t>
   </x:si>
   <x:si>
     <x:t>No catastrophic infinite matching, no timeout errors</x:t>
@@ -38618,8 +38618,8 @@
       <x:c r="BS181" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BT181" t="s">
-        <x:v>1</x:v>
+      <x:c r="BT181" s="6" t="s">
+        <x:v>80</x:v>
       </x:c>
     </x:row>
     <x:row r="182">

</xml_diff>

<commit_message>
Avoid getting version programmatically, with few exceptions. (Reduce start-up time). Update Python engines.
</commit_message>
<xml_diff>
--- a/RegexFeatureMatrix.xlsx
+++ b/RegexFeatureMatrix.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="R4a308b82503f4765"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="R31f2c3925c674661"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -79,7 +79,7 @@
   </x:si>
   <x:si>
     <x:t>Python
- 3.13.6 </x:t>
+ 3.14.5 </x:t>
   </x:si>
   <x:si>
     <x:t>D
@@ -32678,14 +32678,14 @@
       <x:c r="BE136" s="6" t="s">
         <x:v>92</x:v>
       </x:c>
-      <x:c r="BF136" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BG136" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BH136" t="s">
-        <x:v>1</x:v>
+      <x:c r="BF136" s="6" t="s">
+        <x:v>92</x:v>
+      </x:c>
+      <x:c r="BG136" s="6" t="s">
+        <x:v>92</x:v>
+      </x:c>
+      <x:c r="BH136" s="6" t="s">
+        <x:v>92</x:v>
       </x:c>
       <x:c r="BI136" t="s">
         <x:v>1</x:v>
@@ -41795,14 +41795,14 @@
       <x:c r="BQ175" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BR175" s="6" t="s">
-        <x:v>92</x:v>
+      <x:c r="BR175" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="BS175" s="6" t="s">
         <x:v>92</x:v>
       </x:c>
-      <x:c r="BT175" s="6" t="s">
-        <x:v>92</x:v>
+      <x:c r="BT175" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="BU175" s="6" t="s">
         <x:v>92</x:v>
@@ -42530,14 +42530,14 @@
       <x:c r="BQ178" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BR178" s="6" t="s">
-        <x:v>92</x:v>
+      <x:c r="BR178" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="BS178" s="6" t="s">
         <x:v>92</x:v>
       </x:c>
-      <x:c r="BT178" s="6" t="s">
-        <x:v>92</x:v>
+      <x:c r="BT178" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="BU178" s="6" t="s">
         <x:v>92</x:v>
@@ -42787,8 +42787,8 @@
       <x:c r="BU179" s="6" t="s">
         <x:v>92</x:v>
       </x:c>
-      <x:c r="BV179" s="6" t="s">
-        <x:v>92</x:v>
+      <x:c r="BV179" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="BW179" t="s">
         <x:v>1</x:v>
@@ -44465,11 +44465,11 @@
       <x:c r="BF187" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BG187" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BH187" t="s">
-        <x:v>1</x:v>
+      <x:c r="BG187" s="6" t="s">
+        <x:v>92</x:v>
+      </x:c>
+      <x:c r="BH187" s="6" t="s">
+        <x:v>92</x:v>
       </x:c>
       <x:c r="BI187" t="s">
         <x:v>1</x:v>
@@ -50908,14 +50908,14 @@
       <x:c r="BY215" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BZ215" t="s">
-        <x:v>1</x:v>
+      <x:c r="BZ215" s="6" t="s">
+        <x:v>92</x:v>
       </x:c>
       <x:c r="CA215" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CB215" t="s">
-        <x:v>1</x:v>
+      <x:c r="CB215" s="6" t="s">
+        <x:v>92</x:v>
       </x:c>
       <x:c r="CC215" t="s">
         <x:v>1</x:v>

</xml_diff>

<commit_message>
New engine: Resharp (for Rust) 0.6.11.
</commit_message>
<xml_diff>
--- a/RegexFeatureMatrix.xlsx
+++ b/RegexFeatureMatrix.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="R31f2c3925c674661"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="R14563641f65e468f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -248,10 +248,10 @@
     <x:t>fancy_regex (“u” flag)</x:t>
   </x:si>
   <x:si>
-    <x:t>regress (“u” flag)</x:t>
+    <x:t>regress (“uv” flags)</x:t>
   </x:si>
   <x:si>
-    <x:t>regress (“uv” flags)</x:t>
+    <x:t>resharp (“Full” mode)</x:t>
   </x:si>
   <x:si>
     <x:t>regex</x:t>
@@ -1534,8 +1534,8 @@
     <x:col min="51" max="51" width="13.791" customWidth="1"/>
     <x:col min="52" max="52" width="9.796" customWidth="1"/>
     <x:col min="53" max="53" width="19.089" customWidth="1"/>
-    <x:col min="54" max="54" width="15.288" customWidth="1"/>
-    <x:col min="55" max="55" width="17.087" customWidth="1"/>
+    <x:col min="54" max="54" width="17.087" customWidth="1"/>
+    <x:col min="55" max="55" width="18.884" customWidth="1"/>
     <x:col min="56" max="56" width="6.498" customWidth="1"/>
     <x:col min="57" max="57" width="4.998" customWidth="1"/>
     <x:col min="58" max="58" width="3.599" customWidth="1"/>
@@ -3948,8 +3948,8 @@
       <x:c r="BB12" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BC12" t="s">
-        <x:v>1</x:v>
+      <x:c r="BC12" s="6" t="s">
+        <x:v>92</x:v>
       </x:c>
       <x:c r="BD12" s="6" t="s">
         <x:v>92</x:v>
@@ -4438,8 +4438,8 @@
       <x:c r="BB14" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BC14" t="s">
-        <x:v>1</x:v>
+      <x:c r="BC14" s="6" t="s">
+        <x:v>92</x:v>
       </x:c>
       <x:c r="BD14" s="6" t="s">
         <x:v>92</x:v>
@@ -4683,8 +4683,8 @@
       <x:c r="BB15" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BC15" t="s">
-        <x:v>1</x:v>
+      <x:c r="BC15" s="6" t="s">
+        <x:v>92</x:v>
       </x:c>
       <x:c r="BD15" s="6" t="s">
         <x:v>92</x:v>
@@ -5663,8 +5663,8 @@
       <x:c r="BB19" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BC19" t="s">
-        <x:v>1</x:v>
+      <x:c r="BC19" s="6" t="s">
+        <x:v>92</x:v>
       </x:c>
       <x:c r="BD19" s="6" t="s">
         <x:v>92</x:v>
@@ -6640,11 +6640,11 @@
       <x:c r="BA23" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BB23" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BC23" s="6" t="s">
-        <x:v>92</x:v>
+      <x:c r="BB23" s="6" t="s">
+        <x:v>92</x:v>
+      </x:c>
+      <x:c r="BC23" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="BD23" t="s">
         <x:v>1</x:v>
@@ -8856,8 +8856,8 @@
       <x:c r="BB33" s="6" t="s">
         <x:v>92</x:v>
       </x:c>
-      <x:c r="BC33" s="6" t="s">
-        <x:v>92</x:v>
+      <x:c r="BC33" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="BD33" s="6" t="s">
         <x:v>92</x:v>
@@ -9109,8 +9109,8 @@
       <x:c r="BB35" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BC35" t="s">
-        <x:v>1</x:v>
+      <x:c r="BC35" s="6" t="s">
+        <x:v>92</x:v>
       </x:c>
       <x:c r="BD35" s="6" t="s">
         <x:v>92</x:v>
@@ -12294,8 +12294,8 @@
       <x:c r="BB48" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BC48" t="s">
-        <x:v>1</x:v>
+      <x:c r="BC48" s="6" t="s">
+        <x:v>92</x:v>
       </x:c>
       <x:c r="BD48" s="6" t="s">
         <x:v>92</x:v>
@@ -12784,8 +12784,8 @@
       <x:c r="BB50" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BC50" t="s">
-        <x:v>1</x:v>
+      <x:c r="BC50" s="6" t="s">
+        <x:v>92</x:v>
       </x:c>
       <x:c r="BD50" t="s">
         <x:v>1</x:v>
@@ -13274,8 +13274,8 @@
       <x:c r="BB52" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BC52" t="s">
-        <x:v>1</x:v>
+      <x:c r="BC52" s="6" t="s">
+        <x:v>92</x:v>
       </x:c>
       <x:c r="BD52" t="s">
         <x:v>1</x:v>
@@ -13519,8 +13519,8 @@
       <x:c r="BB53" s="6" t="s">
         <x:v>92</x:v>
       </x:c>
-      <x:c r="BC53" s="6" t="s">
-        <x:v>92</x:v>
+      <x:c r="BC53" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="BD53" s="6" t="s">
         <x:v>92</x:v>
@@ -14752,8 +14752,8 @@
       <x:c r="BB59" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BC59" t="s">
-        <x:v>1</x:v>
+      <x:c r="BC59" s="6" t="s">
+        <x:v>92</x:v>
       </x:c>
       <x:c r="BD59" s="6" t="s">
         <x:v>92</x:v>
@@ -14994,8 +14994,8 @@
       <x:c r="BA60" s="6" t="s">
         <x:v>92</x:v>
       </x:c>
-      <x:c r="BB60" s="6" t="s">
-        <x:v>92</x:v>
+      <x:c r="BB60" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="BC60" t="s">
         <x:v>1</x:v>
@@ -17937,8 +17937,8 @@
       <x:c r="BB72" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BC72" t="s">
-        <x:v>1</x:v>
+      <x:c r="BC72" s="6" t="s">
+        <x:v>92</x:v>
       </x:c>
       <x:c r="BD72" s="6" t="s">
         <x:v>92</x:v>
@@ -18427,8 +18427,8 @@
       <x:c r="BB74" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BC74" t="s">
-        <x:v>1</x:v>
+      <x:c r="BC74" s="6" t="s">
+        <x:v>92</x:v>
       </x:c>
       <x:c r="BD74" t="s">
         <x:v>1</x:v>
@@ -18917,8 +18917,8 @@
       <x:c r="BB76" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BC76" t="s">
-        <x:v>1</x:v>
+      <x:c r="BC76" s="6" t="s">
+        <x:v>92</x:v>
       </x:c>
       <x:c r="BD76" t="s">
         <x:v>1</x:v>
@@ -19162,8 +19162,8 @@
       <x:c r="BB77" s="6" t="s">
         <x:v>92</x:v>
       </x:c>
-      <x:c r="BC77" s="6" t="s">
-        <x:v>92</x:v>
+      <x:c r="BC77" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="BD77" s="6" t="s">
         <x:v>92</x:v>
@@ -24315,8 +24315,8 @@
       <x:c r="BB99" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BC99" t="s">
-        <x:v>1</x:v>
+      <x:c r="BC99" s="6" t="s">
+        <x:v>92</x:v>
       </x:c>
       <x:c r="BD99" s="6" t="s">
         <x:v>92</x:v>
@@ -27508,8 +27508,8 @@
       <x:c r="BB113" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BC113" t="s">
-        <x:v>1</x:v>
+      <x:c r="BC113" s="6" t="s">
+        <x:v>92</x:v>
       </x:c>
       <x:c r="BD113" s="6" t="s">
         <x:v>92</x:v>
@@ -27998,8 +27998,8 @@
       <x:c r="BB115" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BC115" t="s">
-        <x:v>1</x:v>
+      <x:c r="BC115" s="6" t="s">
+        <x:v>92</x:v>
       </x:c>
       <x:c r="BD115" t="s">
         <x:v>1</x:v>
@@ -28738,11 +28738,11 @@
       <x:c r="BA119" s="6" t="s">
         <x:v>92</x:v>
       </x:c>
-      <x:c r="BB119" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BC119" s="6" t="s">
-        <x:v>92</x:v>
+      <x:c r="BB119" s="6" t="s">
+        <x:v>92</x:v>
+      </x:c>
+      <x:c r="BC119" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="BD119" s="6" t="s">
         <x:v>92</x:v>
@@ -30698,11 +30698,11 @@
       <x:c r="BA127" s="6" t="s">
         <x:v>92</x:v>
       </x:c>
-      <x:c r="BB127" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BC127" s="6" t="s">
-        <x:v>92</x:v>
+      <x:c r="BB127" s="6" t="s">
+        <x:v>92</x:v>
+      </x:c>
+      <x:c r="BC127" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="BD127" s="6" t="s">
         <x:v>92</x:v>
@@ -31188,11 +31188,11 @@
       <x:c r="BA129" s="6" t="s">
         <x:v>92</x:v>
       </x:c>
-      <x:c r="BB129" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BC129" s="6" t="s">
-        <x:v>92</x:v>
+      <x:c r="BB129" s="6" t="s">
+        <x:v>92</x:v>
+      </x:c>
+      <x:c r="BC129" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="BD129" t="s">
         <x:v>1</x:v>
@@ -32179,8 +32179,8 @@
       <x:c r="BB134" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BC134" t="s">
-        <x:v>1</x:v>
+      <x:c r="BC134" s="6" t="s">
+        <x:v>92</x:v>
       </x:c>
       <x:c r="BD134" s="6" t="s">
         <x:v>92</x:v>
@@ -32669,8 +32669,8 @@
       <x:c r="BB136" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BC136" t="s">
-        <x:v>1</x:v>
+      <x:c r="BC136" s="6" t="s">
+        <x:v>92</x:v>
       </x:c>
       <x:c r="BD136" s="6" t="s">
         <x:v>92</x:v>
@@ -35617,8 +35617,8 @@
       <x:c r="BB149" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BC149" t="s">
-        <x:v>1</x:v>
+      <x:c r="BC149" s="6" t="s">
+        <x:v>92</x:v>
       </x:c>
       <x:c r="BD149" t="s">
         <x:v>1</x:v>
@@ -36107,8 +36107,8 @@
       <x:c r="BB151" s="6" t="s">
         <x:v>92</x:v>
       </x:c>
-      <x:c r="BC151" s="6" t="s">
-        <x:v>92</x:v>
+      <x:c r="BC151" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="BD151" t="s">
         <x:v>1</x:v>
@@ -36352,8 +36352,8 @@
       <x:c r="BB152" s="6" t="s">
         <x:v>92</x:v>
       </x:c>
-      <x:c r="BC152" s="6" t="s">
-        <x:v>92</x:v>
+      <x:c r="BC152" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="BD152" s="6" t="s">
         <x:v>92</x:v>
@@ -36597,8 +36597,8 @@
       <x:c r="BB153" s="6" t="s">
         <x:v>92</x:v>
       </x:c>
-      <x:c r="BC153" s="6" t="s">
-        <x:v>92</x:v>
+      <x:c r="BC153" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="BD153" s="6" t="s">
         <x:v>92</x:v>
@@ -37087,8 +37087,8 @@
       <x:c r="BB155" s="6" t="s">
         <x:v>92</x:v>
       </x:c>
-      <x:c r="BC155" s="6" t="s">
-        <x:v>92</x:v>
+      <x:c r="BC155" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="BD155" s="6" t="s">
         <x:v>92</x:v>
@@ -41505,8 +41505,8 @@
       <x:c r="BB174" s="6" t="s">
         <x:v>92</x:v>
       </x:c>
-      <x:c r="BC174" s="6" t="s">
-        <x:v>92</x:v>
+      <x:c r="BC174" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="BD174" s="6" t="s">
         <x:v>92</x:v>
@@ -41750,8 +41750,8 @@
       <x:c r="BB175" s="6" t="s">
         <x:v>92</x:v>
       </x:c>
-      <x:c r="BC175" s="6" t="s">
-        <x:v>92</x:v>
+      <x:c r="BC175" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="BD175" s="6" t="s">
         <x:v>92</x:v>
@@ -41995,8 +41995,8 @@
       <x:c r="BB176" s="6" t="s">
         <x:v>92</x:v>
       </x:c>
-      <x:c r="BC176" s="6" t="s">
-        <x:v>92</x:v>
+      <x:c r="BC176" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="BD176" s="6" t="s">
         <x:v>92</x:v>
@@ -42240,8 +42240,8 @@
       <x:c r="BB177" s="6" t="s">
         <x:v>92</x:v>
       </x:c>
-      <x:c r="BC177" s="6" t="s">
-        <x:v>92</x:v>
+      <x:c r="BC177" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="BD177" s="6" t="s">
         <x:v>92</x:v>
@@ -42485,8 +42485,8 @@
       <x:c r="BB178" s="6" t="s">
         <x:v>92</x:v>
       </x:c>
-      <x:c r="BC178" s="6" t="s">
-        <x:v>92</x:v>
+      <x:c r="BC178" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="BD178" s="6" t="s">
         <x:v>92</x:v>
@@ -42730,8 +42730,8 @@
       <x:c r="BB179" s="6" t="s">
         <x:v>92</x:v>
       </x:c>
-      <x:c r="BC179" s="6" t="s">
-        <x:v>92</x:v>
+      <x:c r="BC179" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="BD179" s="6" t="s">
         <x:v>92</x:v>
@@ -49124,8 +49124,8 @@
       <x:c r="BB208" s="6" t="s">
         <x:v>92</x:v>
       </x:c>
-      <x:c r="BC208" s="6" t="s">
-        <x:v>92</x:v>
+      <x:c r="BC208" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="BD208" t="s">
         <x:v>1</x:v>
@@ -49369,8 +49369,8 @@
       <x:c r="BB209" s="6" t="s">
         <x:v>92</x:v>
       </x:c>
-      <x:c r="BC209" s="6" t="s">
-        <x:v>92</x:v>
+      <x:c r="BC209" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="BD209" t="s">
         <x:v>1</x:v>
@@ -50349,8 +50349,8 @@
       <x:c r="BB213" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BC213" t="s">
-        <x:v>1</x:v>
+      <x:c r="BC213" s="6" t="s">
+        <x:v>92</x:v>
       </x:c>
       <x:c r="BD213" s="6" t="s">
         <x:v>92</x:v>
@@ -52072,8 +52072,8 @@
       <x:c r="BB221" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BC221" t="s">
-        <x:v>1</x:v>
+      <x:c r="BC221" s="6" t="s">
+        <x:v>92</x:v>
       </x:c>
       <x:c r="BD221" t="s">
         <x:v>1</x:v>
@@ -52317,8 +52317,8 @@
       <x:c r="BB222" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BC222" t="s">
-        <x:v>1</x:v>
+      <x:c r="BC222" s="6" t="s">
+        <x:v>92</x:v>
       </x:c>
       <x:c r="BD222" t="s">
         <x:v>1</x:v>
@@ -52562,8 +52562,8 @@
       <x:c r="BB223" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BC223" t="s">
-        <x:v>1</x:v>
+      <x:c r="BC223" s="6" t="s">
+        <x:v>92</x:v>
       </x:c>
       <x:c r="BD223" t="s">
         <x:v>1</x:v>

</xml_diff>

<commit_message>
Update ANRE engine: 2.1.1.
</commit_message>
<xml_diff>
--- a/RegexFeatureMatrix.xlsx
+++ b/RegexFeatureMatrix.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="Rd5219d3dd367459b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="R4e6c79aab5344f2a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1360,6 +1360,9 @@
   <x:si>
     <x:t>Complement (pattern must not match)</x:t>
   </x:si>
+  <x:si>
+    <x:t>Also supports alternative syntax</x:t>
+  </x:si>
 </x:sst>
 </file>
 
@@ -36773,8 +36776,8 @@
       <x:c r="AZ152" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BA152" t="s">
-        <x:v>1</x:v>
+      <x:c r="BA152" s="6" t="s">
+        <x:v>93</x:v>
       </x:c>
       <x:c r="BB152" s="6" t="s">
         <x:v>93</x:v>
@@ -37021,8 +37024,8 @@
       <x:c r="AZ153" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BA153" t="s">
-        <x:v>1</x:v>
+      <x:c r="BA153" s="6" t="s">
+        <x:v>93</x:v>
       </x:c>
       <x:c r="BB153" s="6" t="s">
         <x:v>93</x:v>
@@ -48124,8 +48127,8 @@
       <x:c r="Y201" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="Z201" t="s">
-        <x:v>1</x:v>
+      <x:c r="Z201" s="6" t="s">
+        <x:v>93</x:v>
       </x:c>
       <x:c r="AA201" t="s">
         <x:v>1</x:v>
@@ -48151,8 +48154,8 @@
       <x:c r="AH201" s="6" t="s">
         <x:v>93</x:v>
       </x:c>
-      <x:c r="AI201" t="s">
-        <x:v>1</x:v>
+      <x:c r="AI201" s="6" t="s">
+        <x:v>93</x:v>
       </x:c>
       <x:c r="AJ201" t="s">
         <x:v>1</x:v>
@@ -48175,8 +48178,8 @@
       <x:c r="AP201" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="AQ201" t="s">
-        <x:v>1</x:v>
+      <x:c r="AQ201" s="6" t="s">
+        <x:v>93</x:v>
       </x:c>
       <x:c r="AR201" t="s">
         <x:v>1</x:v>
@@ -48196,8 +48199,8 @@
       <x:c r="AW201" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="AX201" t="s">
-        <x:v>1</x:v>
+      <x:c r="AX201" s="6" t="s">
+        <x:v>93</x:v>
       </x:c>
       <x:c r="AY201" t="s">
         <x:v>1</x:v>
@@ -53273,250 +53276,498 @@
       </x:c>
     </x:row>
     <x:row r="224">
-      <x:c r="A224" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="B224" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C224" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D224" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E224" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F224" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G224" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="H224" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I224" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="J224" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="K224" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="L224" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="M224" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="N224" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="O224" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="P224" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="Q224" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="R224" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="S224" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="T224" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="U224" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="V224" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="W224" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="X224" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="Y224" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="Z224" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AA224" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AB224" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AC224" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AD224" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AE224" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AF224" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AG224" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AH224" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AI224" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AJ224" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AK224" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AL224" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AM224" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AN224" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AO224" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AP224" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AQ224" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AR224" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AS224" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AT224" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AU224" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AV224" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AW224" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AX224" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AY224" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AZ224" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BA224" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BB224" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BC224" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BD224" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BE224" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BF224" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BG224" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BH224" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BI224" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BJ224" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BK224" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BL224" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BM224" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BN224" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BO224" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BP224" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BQ224" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BR224" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BS224" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BT224" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BU224" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BV224" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BW224" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BX224" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BY224" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BZ224" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CA224" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CB224" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CC224" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CD224" s="7" t="s">
+      <x:c r="A224" s="4" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B224" s="5" t="s">
+        <x:v>441</x:v>
+      </x:c>
+      <x:c r="C224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="O224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Q224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="R224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="S224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="T224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="V224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="W224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="X224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Y224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Z224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AA224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AB224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AC224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AD224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AE224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AF224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AG224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AH224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AI224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AJ224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AK224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AL224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AM224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AN224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AO224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AP224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AQ224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AR224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AS224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AT224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AU224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AV224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AW224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AX224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AY224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AZ224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BA224" s="6" t="s">
+        <x:v>93</x:v>
+      </x:c>
+      <x:c r="BB224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BC224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BD224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BE224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BF224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BG224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BH224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BI224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BJ224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BK224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BL224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BM224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BN224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BO224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BP224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BQ224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BR224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BS224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BT224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BU224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BV224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BW224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BX224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BY224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BZ224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CA224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CB224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CC224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CD224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="225">
+      <x:c r="A225" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B225" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C225" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D225" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E225" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F225" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G225" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H225" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I225" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J225" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K225" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L225" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M225" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N225" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="O225" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P225" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Q225" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="R225" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="S225" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="T225" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U225" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="V225" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="W225" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="X225" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Y225" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Z225" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AA225" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AB225" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AC225" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AD225" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AE225" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AF225" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AG225" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AH225" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AI225" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AJ225" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AK225" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AL225" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AM225" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AN225" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AO225" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AP225" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AQ225" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AR225" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AS225" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AT225" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AU225" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AV225" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AW225" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AX225" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AY225" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AZ225" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BA225" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BB225" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BC225" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BD225" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BE225" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BF225" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BG225" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BH225" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BI225" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BJ225" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BK225" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BL225" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BM225" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BN225" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BO225" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BP225" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BQ225" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BR225" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BS225" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BT225" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BU225" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BV225" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BW225" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BX225" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BY225" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BZ225" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CA225" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CB225" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CC225" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CD225" s="7" t="s">
         <x:v>1</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Update REAL engines (C++ and Python): 2026.7.2.
</commit_message>
<xml_diff>
--- a/RegexFeatureMatrix.xlsx
+++ b/RegexFeatureMatrix.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="R684a899600e54427"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="R18bb6aefb12f482d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -139,7 +139,7 @@
   </x:si>
   <x:si>
     <x:t>REAL
- 2026.6.21 </x:t>
+ 2026.7.2 </x:t>
   </x:si>
   <x:si>
     <x:t>ECMAScript</x:t>
@@ -1600,7 +1600,7 @@
     <x:col min="82" max="82" width="14.292" customWidth="1"/>
     <x:col min="83" max="83" width="8.396" customWidth="1"/>
     <x:col min="84" max="84" width="16.391" customWidth="1"/>
-    <x:col min="85" max="85" width="11" customWidth="1"/>
+    <x:col min="85" max="85" width="10" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="49" customHeight="1">
@@ -52262,8 +52262,8 @@
       <x:c r="BF211" s="6" t="s">
         <x:v>97</x:v>
       </x:c>
-      <x:c r="BG211" t="s">
-        <x:v>1</x:v>
+      <x:c r="BG211" s="6" t="s">
+        <x:v>97</x:v>
       </x:c>
       <x:c r="BH211" s="6" t="s">
         <x:v>97</x:v>
@@ -52340,8 +52340,8 @@
       <x:c r="CF211" s="6" t="s">
         <x:v>97</x:v>
       </x:c>
-      <x:c r="CG211" t="s">
-        <x:v>1</x:v>
+      <x:c r="CG211" s="6" t="s">
+        <x:v>97</x:v>
       </x:c>
     </x:row>
     <x:row r="212">
@@ -52519,8 +52519,8 @@
       <x:c r="BF212" s="6" t="s">
         <x:v>97</x:v>
       </x:c>
-      <x:c r="BG212" t="s">
-        <x:v>1</x:v>
+      <x:c r="BG212" s="6" t="s">
+        <x:v>97</x:v>
       </x:c>
       <x:c r="BH212" s="6" t="s">
         <x:v>97</x:v>
@@ -52597,8 +52597,8 @@
       <x:c r="CF212" s="6" t="s">
         <x:v>97</x:v>
       </x:c>
-      <x:c r="CG212" t="s">
-        <x:v>1</x:v>
+      <x:c r="CG212" s="6" t="s">
+        <x:v>97</x:v>
       </x:c>
     </x:row>
     <x:row r="213">
@@ -53804,8 +53804,8 @@
       <x:c r="BF217" s="6" t="s">
         <x:v>97</x:v>
       </x:c>
-      <x:c r="BG217" t="s">
-        <x:v>1</x:v>
+      <x:c r="BG217" s="6" t="s">
+        <x:v>97</x:v>
       </x:c>
       <x:c r="BH217" s="6" t="s">
         <x:v>97</x:v>
@@ -53882,8 +53882,8 @@
       <x:c r="CF217" s="6" t="s">
         <x:v>97</x:v>
       </x:c>
-      <x:c r="CG217" t="s">
-        <x:v>1</x:v>
+      <x:c r="CG217" s="6" t="s">
+        <x:v>97</x:v>
       </x:c>
     </x:row>
     <x:row r="218">

</xml_diff>

<commit_message>
Update REAL engines (C++ and Python): 2026.7.3.
</commit_message>
<xml_diff>
--- a/RegexFeatureMatrix.xlsx
+++ b/RegexFeatureMatrix.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="R56c98883c66c45d2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="Rcd9aabf843854d38"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -139,7 +139,7 @@
   </x:si>
   <x:si>
     <x:t>REAL
- 2026.7.2 </x:t>
+ 2026.7.3 </x:t>
   </x:si>
   <x:si>
     <x:t>ECMAScript</x:t>
@@ -27283,8 +27283,8 @@
       <x:c r="BF107" s="6" t="s">
         <x:v>97</x:v>
       </x:c>
-      <x:c r="BG107" t="s">
-        <x:v>1</x:v>
+      <x:c r="BG107" s="6" t="s">
+        <x:v>97</x:v>
       </x:c>
       <x:c r="BH107" s="6" t="s">
         <x:v>97</x:v>
@@ -27361,8 +27361,8 @@
       <x:c r="CF107" s="6" t="s">
         <x:v>97</x:v>
       </x:c>
-      <x:c r="CG107" t="s">
-        <x:v>1</x:v>
+      <x:c r="CG107" s="6" t="s">
+        <x:v>97</x:v>
       </x:c>
     </x:row>
     <x:row r="108">

</xml_diff>

<commit_message>
Update REAL engines (C++ and Python): 2026.7.8.
</commit_message>
<xml_diff>
--- a/RegexFeatureMatrix.xlsx
+++ b/RegexFeatureMatrix.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="R2f77761af6c54fc8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="R567d64d94c3f45b1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -139,7 +139,7 @@
   </x:si>
   <x:si>
     <x:t>REAL
- 2026.7.3 </x:t>
+ 2026.7.8 </x:t>
   </x:si>
   <x:si>
     <x:t>ECMAScript</x:t>
@@ -5141,8 +5141,8 @@
       <x:c r="BF16" s="6" t="s">
         <x:v>97</x:v>
       </x:c>
-      <x:c r="BG16" t="s">
-        <x:v>1</x:v>
+      <x:c r="BG16" s="6" t="s">
+        <x:v>97</x:v>
       </x:c>
       <x:c r="BH16" t="s">
         <x:v>1</x:v>
@@ -5219,8 +5219,8 @@
       <x:c r="CF16" s="6" t="s">
         <x:v>97</x:v>
       </x:c>
-      <x:c r="CG16" t="s">
-        <x:v>1</x:v>
+      <x:c r="CG16" s="6" t="s">
+        <x:v>97</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -14923,8 +14923,8 @@
       <x:c r="BF56" s="6" t="s">
         <x:v>97</x:v>
       </x:c>
-      <x:c r="BG56" t="s">
-        <x:v>1</x:v>
+      <x:c r="BG56" s="6" t="s">
+        <x:v>97</x:v>
       </x:c>
       <x:c r="BH56" t="s">
         <x:v>1</x:v>
@@ -15001,8 +15001,8 @@
       <x:c r="CF56" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CG56" t="s">
-        <x:v>1</x:v>
+      <x:c r="CG56" s="6" t="s">
+        <x:v>97</x:v>
       </x:c>
     </x:row>
     <x:row r="57">
@@ -17501,8 +17501,8 @@
       <x:c r="BF67" s="6" t="s">
         <x:v>97</x:v>
       </x:c>
-      <x:c r="BG67" t="s">
-        <x:v>1</x:v>
+      <x:c r="BG67" s="6" t="s">
+        <x:v>97</x:v>
       </x:c>
       <x:c r="BH67" t="s">
         <x:v>1</x:v>
@@ -17579,8 +17579,8 @@
       <x:c r="CF67" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CG67" t="s">
-        <x:v>1</x:v>
+      <x:c r="CG67" s="6" t="s">
+        <x:v>97</x:v>
       </x:c>
     </x:row>
     <x:row r="68">
@@ -17758,8 +17758,8 @@
       <x:c r="BF68" s="6" t="s">
         <x:v>97</x:v>
       </x:c>
-      <x:c r="BG68" t="s">
-        <x:v>1</x:v>
+      <x:c r="BG68" s="6" t="s">
+        <x:v>97</x:v>
       </x:c>
       <x:c r="BH68" t="s">
         <x:v>1</x:v>
@@ -17836,8 +17836,8 @@
       <x:c r="CF68" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CG68" t="s">
-        <x:v>1</x:v>
+      <x:c r="CG68" s="6" t="s">
+        <x:v>97</x:v>
       </x:c>
     </x:row>
     <x:row r="69">
@@ -20842,8 +20842,8 @@
       <x:c r="BF80" s="6" t="s">
         <x:v>97</x:v>
       </x:c>
-      <x:c r="BG80" t="s">
-        <x:v>1</x:v>
+      <x:c r="BG80" s="6" t="s">
+        <x:v>97</x:v>
       </x:c>
       <x:c r="BH80" t="s">
         <x:v>1</x:v>
@@ -20920,8 +20920,8 @@
       <x:c r="CF80" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CG80" t="s">
-        <x:v>1</x:v>
+      <x:c r="CG80" s="6" t="s">
+        <x:v>97</x:v>
       </x:c>
     </x:row>
     <x:row r="81">
@@ -34238,8 +34238,8 @@
       <x:c r="BF136" s="6" t="s">
         <x:v>97</x:v>
       </x:c>
-      <x:c r="BG136" t="s">
-        <x:v>1</x:v>
+      <x:c r="BG136" s="6" t="s">
+        <x:v>97</x:v>
       </x:c>
       <x:c r="BH136" t="s">
         <x:v>1</x:v>
@@ -34316,8 +34316,8 @@
       <x:c r="CF136" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CG136" t="s">
-        <x:v>1</x:v>
+      <x:c r="CG136" s="6" t="s">
+        <x:v>97</x:v>
       </x:c>
     </x:row>
     <x:row r="137">

</xml_diff>

<commit_message>
Update REAL engines (C++ and Python): 2026.7.19.
</commit_message>
<xml_diff>
--- a/RegexFeatureMatrix.xlsx
+++ b/RegexFeatureMatrix.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="R567d64d94c3f45b1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="R73b7c57dbab74ed4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -127,7 +127,7 @@
   </x:si>
   <x:si>
     <x:t>RE#
- 1.0.3 </x:t>
+ 1.0.4 </x:t>
   </x:si>
   <x:si>
     <x:t>Go
@@ -139,7 +139,7 @@
   </x:si>
   <x:si>
     <x:t>REAL
- 2026.7.8 </x:t>
+ 2026.7.19 </x:t>
   </x:si>
   <x:si>
     <x:t>ECMAScript</x:t>
@@ -1606,7 +1606,7 @@
     <x:col min="82" max="82" width="14.292" customWidth="1"/>
     <x:col min="83" max="83" width="8.396" customWidth="1"/>
     <x:col min="84" max="84" width="16.391" customWidth="1"/>
-    <x:col min="85" max="85" width="10" customWidth="1"/>
+    <x:col min="85" max="85" width="11" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="49" customHeight="1">

</xml_diff>

<commit_message>
Update REAL engines (C++, Python, Rust): 2026..7.21.
</commit_message>
<xml_diff>
--- a/RegexFeatureMatrix.xlsx
+++ b/RegexFeatureMatrix.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="Ref08a4a068424e99"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="R53155b3bc2554f0c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -139,7 +139,7 @@
   </x:si>
   <x:si>
     <x:t>REAL
- 2026.7.19 </x:t>
+ 2026.7.21 </x:t>
   </x:si>
   <x:si>
     <x:t>ECMAScript</x:t>

</xml_diff>

<commit_message>
Update RE2JS engine: 2.8.6. Clarify Feature Matrix.
</commit_message>
<xml_diff>
--- a/RegexFeatureMatrix.xlsx
+++ b/RegexFeatureMatrix.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="R53155b3bc2554f0c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="Rc75ce961ede14db9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -15113,8 +15113,8 @@
       <x:c r="BR56" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BS56" t="s">
-        <x:v>1</x:v>
+      <x:c r="BS56" s="6" t="s">
+        <x:v>97</x:v>
       </x:c>
       <x:c r="BT56" t="s">
         <x:v>1</x:v>
@@ -21101,8 +21101,8 @@
       <x:c r="BR80" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BS80" t="s">
-        <x:v>1</x:v>
+      <x:c r="BS80" s="6" t="s">
+        <x:v>97</x:v>
       </x:c>
       <x:c r="BT80" t="s">
         <x:v>1</x:v>

</xml_diff>

<commit_message>
Update REAL engines (C++, Python, Rust): 2026.7.23.
</commit_message>
<xml_diff>
--- a/RegexFeatureMatrix.xlsx
+++ b/RegexFeatureMatrix.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="Rc75ce961ede14db9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="R79afd2ead30442d5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -139,7 +139,7 @@
   </x:si>
   <x:si>
     <x:t>REAL
- 2026.7.21 </x:t>
+ 2026.7.23 </x:t>
   </x:si>
   <x:si>
     <x:t>ECMAScript</x:t>
@@ -25738,8 +25738,8 @@
       <x:c r="BA99" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BB99" t="s">
-        <x:v>1</x:v>
+      <x:c r="BB99" s="6" t="s">
+        <x:v>97</x:v>
       </x:c>
       <x:c r="BC99" s="6" t="s">
         <x:v>97</x:v>
@@ -25756,8 +25756,8 @@
       <x:c r="BG99" s="6" t="s">
         <x:v>97</x:v>
       </x:c>
-      <x:c r="BH99" t="s">
-        <x:v>1</x:v>
+      <x:c r="BH99" s="6" t="s">
+        <x:v>97</x:v>
       </x:c>
       <x:c r="BI99" s="6" t="s">
         <x:v>97</x:v>
@@ -25834,8 +25834,8 @@
       <x:c r="CG99" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CH99" t="s">
-        <x:v>1</x:v>
+      <x:c r="CH99" s="6" t="s">
+        <x:v>97</x:v>
       </x:c>
     </x:row>
     <x:row r="100">
@@ -25998,8 +25998,8 @@
       <x:c r="BA100" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BB100" t="s">
-        <x:v>1</x:v>
+      <x:c r="BB100" s="6" t="s">
+        <x:v>97</x:v>
       </x:c>
       <x:c r="BC100" s="6" t="s">
         <x:v>97</x:v>
@@ -26016,8 +26016,8 @@
       <x:c r="BG100" s="6" t="s">
         <x:v>97</x:v>
       </x:c>
-      <x:c r="BH100" t="s">
-        <x:v>1</x:v>
+      <x:c r="BH100" s="6" t="s">
+        <x:v>97</x:v>
       </x:c>
       <x:c r="BI100" s="6" t="s">
         <x:v>97</x:v>
@@ -26094,8 +26094,8 @@
       <x:c r="CG100" s="6" t="s">
         <x:v>97</x:v>
       </x:c>
-      <x:c r="CH100" t="s">
-        <x:v>1</x:v>
+      <x:c r="CH100" s="6" t="s">
+        <x:v>97</x:v>
       </x:c>
     </x:row>
     <x:row r="101">
@@ -29126,8 +29126,8 @@
       <x:c r="BA113" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BB113" t="s">
-        <x:v>1</x:v>
+      <x:c r="BB113" s="6" t="s">
+        <x:v>97</x:v>
       </x:c>
       <x:c r="BC113" s="6" t="s">
         <x:v>97</x:v>
@@ -29144,8 +29144,8 @@
       <x:c r="BG113" s="6" t="s">
         <x:v>97</x:v>
       </x:c>
-      <x:c r="BH113" t="s">
-        <x:v>1</x:v>
+      <x:c r="BH113" s="6" t="s">
+        <x:v>97</x:v>
       </x:c>
       <x:c r="BI113" s="6" t="s">
         <x:v>97</x:v>
@@ -29222,8 +29222,8 @@
       <x:c r="CG113" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CH113" t="s">
-        <x:v>1</x:v>
+      <x:c r="CH113" s="6" t="s">
+        <x:v>97</x:v>
       </x:c>
     </x:row>
     <x:row r="114">
@@ -29386,8 +29386,8 @@
       <x:c r="BA114" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BB114" t="s">
-        <x:v>1</x:v>
+      <x:c r="BB114" s="6" t="s">
+        <x:v>97</x:v>
       </x:c>
       <x:c r="BC114" s="6" t="s">
         <x:v>97</x:v>
@@ -29404,8 +29404,8 @@
       <x:c r="BG114" s="6" t="s">
         <x:v>97</x:v>
       </x:c>
-      <x:c r="BH114" t="s">
-        <x:v>1</x:v>
+      <x:c r="BH114" s="6" t="s">
+        <x:v>97</x:v>
       </x:c>
       <x:c r="BI114" s="6" t="s">
         <x:v>97</x:v>
@@ -29482,8 +29482,8 @@
       <x:c r="CG114" s="6" t="s">
         <x:v>97</x:v>
       </x:c>
-      <x:c r="CH114" t="s">
-        <x:v>1</x:v>
+      <x:c r="CH114" s="6" t="s">
+        <x:v>97</x:v>
       </x:c>
     </x:row>
     <x:row r="115">

</xml_diff>

<commit_message>
Update REAL engines (C++, Python, Rust): 2026.7.25.
</commit_message>
<xml_diff>
--- a/RegexFeatureMatrix.xlsx
+++ b/RegexFeatureMatrix.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="R79afd2ead30442d5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="Rec98bddc357e421f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -139,7 +139,7 @@
   </x:si>
   <x:si>
     <x:t>REAL
- 2026.7.23 </x:t>
+ 2026.7.25 </x:t>
   </x:si>
   <x:si>
     <x:t>ECMAScript</x:t>

</xml_diff>

<commit_message>
Update REAL engines (C++, Python, Rust): 2026.7.26.
</commit_message>
<xml_diff>
--- a/RegexFeatureMatrix.xlsx
+++ b/RegexFeatureMatrix.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="Rec98bddc357e421f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="R467fc079db6947f3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -139,7 +139,7 @@
   </x:si>
   <x:si>
     <x:t>REAL
- 2026.7.25 </x:t>
+ 2026.7.26 </x:t>
   </x:si>
   <x:si>
     <x:t>ECMAScript</x:t>
@@ -1306,19 +1306,19 @@
     <x:t>Unicode</x:t>
   </x:si>
   <x:si>
-    <x:t>Supports Unicode characters, not just ASCII</x:t>
+    <x:t>Support Unicode characters, not just ASCII</x:t>
   </x:si>
   <x:si>
     <x:t>[Unicode]</x:t>
   </x:si>
   <x:si>
-    <x:t>Supports Unicode characters inside sets</x:t>
+    <x:t>Support Unicode characters inside sets</x:t>
   </x:si>
   <x:si>
     <x:t>é=É</x:t>
   </x:si>
   <x:si>
-    <x:t>Supports Unicode case folding</x:t>
+    <x:t>Support Unicode case folding</x:t>
   </x:si>
   <x:si>
     <x:t>Surrogates</x:t>
@@ -1396,7 +1396,7 @@
     <x:t>Get all captures matched by group</x:t>
   </x:si>
   <x:si>
-    <x:t>Also supports alternative syntax</x:t>
+    <x:t>Also support alternative syntax</x:t>
   </x:si>
 </x:sst>
 </file>

</xml_diff>

<commit_message>
Update REAL engines (C++, Python, Rust): 2026.7.40.
</commit_message>
<xml_diff>
--- a/RegexFeatureMatrix.xlsx
+++ b/RegexFeatureMatrix.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="R05e2d5b06e1042fc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="R30364a5351814b4d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -139,7 +139,7 @@
   </x:si>
   <x:si>
     <x:t>REAL
- 2026.7.35 </x:t>
+ 2026.7.40 </x:t>
   </x:si>
   <x:si>
     <x:t>ECMAScript</x:t>

</xml_diff>

<commit_message>
Update REAL engines (C++, Python, Rust): 2026.7.46.
</commit_message>
<xml_diff>
--- a/RegexFeatureMatrix.xlsx
+++ b/RegexFeatureMatrix.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="R30364a5351814b4d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="R785ce283f1434f37"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -23,7 +23,7 @@
   </x:si>
   <x:si>
     <x:t>.NET
- 9.0.17 </x:t>
+ 9.0.18 </x:t>
   </x:si>
   <x:si>
     <x:t>wregex
@@ -139,7 +139,7 @@
   </x:si>
   <x:si>
     <x:t>REAL
- 2026.7.40 </x:t>
+ 2026.7.46 </x:t>
   </x:si>
   <x:si>
     <x:t>ECMAScript</x:t>

</xml_diff>

<commit_message>
Update ANRE engine: 2.1.2.
</commit_message>
<xml_diff>
--- a/RegexFeatureMatrix.xlsx
+++ b/RegexFeatureMatrix.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="R785ce283f1434f37"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="R16382bb51d83476f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -139,7 +139,7 @@
   </x:si>
   <x:si>
     <x:t>REAL
- 2026.7.46 </x:t>
+ 2026.7.50 </x:t>
   </x:si>
   <x:si>
     <x:t>ECMAScript</x:t>

</xml_diff>

<commit_message>
Update REAL engines (C++, Python, Rust): 2026.7.51.
</commit_message>
<xml_diff>
--- a/RegexFeatureMatrix.xlsx
+++ b/RegexFeatureMatrix.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="R16382bb51d83476f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="R39961fa6fd3041c9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -139,7 +139,7 @@
   </x:si>
   <x:si>
     <x:t>REAL
- 2026.7.50 </x:t>
+ 2026.7.51 </x:t>
   </x:si>
   <x:si>
     <x:t>ECMAScript</x:t>
@@ -6655,11 +6655,11 @@
       <x:c r="BA21" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BB21" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BC21" t="s">
-        <x:v>1</x:v>
+      <x:c r="BB21" s="6" t="s">
+        <x:v>101</x:v>
+      </x:c>
+      <x:c r="BC21" s="6" t="s">
+        <x:v>101</x:v>
       </x:c>
       <x:c r="BD21" s="6" t="s">
         <x:v>101</x:v>
@@ -6676,11 +6676,11 @@
       <x:c r="BH21" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BI21" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BJ21" t="s">
-        <x:v>1</x:v>
+      <x:c r="BI21" s="6" t="s">
+        <x:v>101</x:v>
+      </x:c>
+      <x:c r="BJ21" s="6" t="s">
+        <x:v>101</x:v>
       </x:c>
       <x:c r="BK21" t="s">
         <x:v>1</x:v>
@@ -6757,11 +6757,11 @@
       <x:c r="CI21" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CJ21" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CK21" t="s">
-        <x:v>1</x:v>
+      <x:c r="CJ21" s="6" t="s">
+        <x:v>101</x:v>
+      </x:c>
+      <x:c r="CK21" s="6" t="s">
+        <x:v>101</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
@@ -13665,11 +13665,11 @@
       <x:c r="BA49" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BB49" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BC49" t="s">
-        <x:v>1</x:v>
+      <x:c r="BB49" s="6" t="s">
+        <x:v>101</x:v>
+      </x:c>
+      <x:c r="BC49" s="6" t="s">
+        <x:v>101</x:v>
       </x:c>
       <x:c r="BD49" s="6" t="s">
         <x:v>101</x:v>
@@ -13686,11 +13686,11 @@
       <x:c r="BH49" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BI49" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BJ49" t="s">
-        <x:v>1</x:v>
+      <x:c r="BI49" s="6" t="s">
+        <x:v>101</x:v>
+      </x:c>
+      <x:c r="BJ49" s="6" t="s">
+        <x:v>101</x:v>
       </x:c>
       <x:c r="BK49" t="s">
         <x:v>1</x:v>
@@ -13767,11 +13767,11 @@
       <x:c r="CI49" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CJ49" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CK49" t="s">
-        <x:v>1</x:v>
+      <x:c r="CJ49" s="6" t="s">
+        <x:v>101</x:v>
+      </x:c>
+      <x:c r="CK49" s="6" t="s">
+        <x:v>101</x:v>
       </x:c>
     </x:row>
     <x:row r="50">
@@ -19860,11 +19860,11 @@
       <x:c r="BA73" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BB73" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BC73" t="s">
-        <x:v>1</x:v>
+      <x:c r="BB73" s="6" t="s">
+        <x:v>101</x:v>
+      </x:c>
+      <x:c r="BC73" s="6" t="s">
+        <x:v>101</x:v>
       </x:c>
       <x:c r="BD73" s="6" t="s">
         <x:v>101</x:v>
@@ -19881,11 +19881,11 @@
       <x:c r="BH73" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BI73" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BJ73" t="s">
-        <x:v>1</x:v>
+      <x:c r="BI73" s="6" t="s">
+        <x:v>101</x:v>
+      </x:c>
+      <x:c r="BJ73" s="6" t="s">
+        <x:v>101</x:v>
       </x:c>
       <x:c r="BK73" t="s">
         <x:v>1</x:v>
@@ -19962,11 +19962,11 @@
       <x:c r="CI73" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CJ73" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CK73" t="s">
-        <x:v>1</x:v>
+      <x:c r="CJ73" s="6" t="s">
+        <x:v>101</x:v>
+      </x:c>
+      <x:c r="CK73" s="6" t="s">
+        <x:v>101</x:v>
       </x:c>
     </x:row>
     <x:row r="74">

</xml_diff>

<commit_message>
Update RE# engine: 1.0.5.
</commit_message>
<xml_diff>
--- a/RegexFeatureMatrix.xlsx
+++ b/RegexFeatureMatrix.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="R39961fa6fd3041c9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="R0439f05cf80a4dde"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -127,7 +127,7 @@
   </x:si>
   <x:si>
     <x:t>RE#
- 1.0.4 </x:t>
+ 1.0.5 </x:t>
   </x:si>
   <x:si>
     <x:t>Go
@@ -14547,8 +14547,8 @@
       <x:c r="BZ52" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CA52" t="s">
-        <x:v>1</x:v>
+      <x:c r="CA52" s="6" t="s">
+        <x:v>101</x:v>
       </x:c>
       <x:c r="CB52" t="s">
         <x:v>1</x:v>
@@ -20742,8 +20742,8 @@
       <x:c r="BZ76" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CA76" t="s">
-        <x:v>1</x:v>
+      <x:c r="CA76" s="6" t="s">
+        <x:v>101</x:v>
       </x:c>
       <x:c r="CB76" t="s">
         <x:v>1</x:v>

</xml_diff>

<commit_message>
Update REAL engines (C++, Python, Rust): 2026.7.55.
</commit_message>
<xml_diff>
--- a/RegexFeatureMatrix.xlsx
+++ b/RegexFeatureMatrix.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="R8c31f20cb5fc4f5d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="R5ee06e1429c34c08"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -139,7 +139,7 @@
   </x:si>
   <x:si>
     <x:t>REAL
- 2026.7.51 </x:t>
+ 2026.7.55 </x:t>
   </x:si>
   <x:si>
     <x:t>ECMAScript</x:t>

</xml_diff>

<commit_message>
New Feature Matrix indicator: “ß ↔ ss”. Update REAL engines (C++, Python, Rust): 2026.7.63.
</commit_message>
<xml_diff>
--- a/RegexFeatureMatrix.xlsx
+++ b/RegexFeatureMatrix.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="R7ae56ec95e10415b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="R0aaa27c948b64736"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -139,7 +139,7 @@
   </x:si>
   <x:si>
     <x:t>REAL
- 2026.7.62 </x:t>
+ 2026.7.63 </x:t>
   </x:si>
   <x:si>
     <x:t>ECMAScript</x:t>
@@ -1354,16 +1354,28 @@
     <x:t>Support Unicode characters inside sets</x:t>
   </x:si>
   <x:si>
+    <x:t>Surrogates</x:t>
+  </x:si>
+  <x:si>
+    <x:t>“.” matches surrogate pairs as one entity (no split)</x:t>
+  </x:si>
+  <x:si>
     <x:t>é=É</x:t>
   </x:si>
   <x:si>
     <x:t>Support Unicode case folding</x:t>
   </x:si>
   <x:si>
-    <x:t>Surrogates</x:t>
+    <x:t>Σσς</x:t>
   </x:si>
   <x:si>
-    <x:t>“.” matches surrogate pairs as one entity (no split)</x:t>
+    <x:t>Match letters that have multiple uppercase and lowercase variants</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ß=SS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Match “ß ↔ ss” and “ß ↔ SS” in case-insensitive mode</x:t>
   </x:si>
   <x:si>
     <x:t>Fuzzy matching</x:t>
@@ -1382,12 +1394,6 @@
   </x:si>
   <x:si>
     <x:t>Give error on possible ReDoS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Σσς</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Match letters that have multiple uppercase and lowercase variants</x:t>
   </x:si>
   <x:si>
     <x:t>Specific extensions</x:t>
@@ -57975,8 +57981,8 @@
       <x:c r="B215" s="5" t="s">
         <x:v>439</x:v>
       </x:c>
-      <x:c r="C215" s="6" t="s">
-        <x:v>106</x:v>
+      <x:c r="C215" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D215" t="s">
         <x:v>1</x:v>
@@ -57999,14 +58005,14 @@
       <x:c r="J215" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="K215" s="6" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="L215" s="6" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="M215" s="6" t="s">
-        <x:v>106</x:v>
+      <x:c r="K215" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L215" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M215" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="N215" s="6" t="s">
         <x:v>106</x:v>
@@ -58017,35 +58023,35 @@
       <x:c r="P215" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="Q215" s="6" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="R215" s="6" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="S215" s="6" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="T215" s="6" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="U215" s="6" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="V215" s="6" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="W215" s="6" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="X215" s="6" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="Y215" s="6" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="Z215" s="6" t="s">
-        <x:v>106</x:v>
+      <x:c r="Q215" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="R215" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="S215" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="T215" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U215" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="V215" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="W215" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="X215" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Y215" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Z215" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="AA215" s="6" t="s">
         <x:v>106</x:v>
@@ -58080,8 +58086,8 @@
       <x:c r="AK215" s="6" t="s">
         <x:v>106</x:v>
       </x:c>
-      <x:c r="AL215" s="6" t="s">
-        <x:v>106</x:v>
+      <x:c r="AL215" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="AM215" s="6" t="s">
         <x:v>106</x:v>
@@ -58101,8 +58107,8 @@
       <x:c r="AR215" s="6" t="s">
         <x:v>106</x:v>
       </x:c>
-      <x:c r="AS215" s="6" t="s">
-        <x:v>106</x:v>
+      <x:c r="AS215" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="AT215" s="6" t="s">
         <x:v>106</x:v>
@@ -58116,8 +58122,8 @@
       <x:c r="AW215" s="6" t="s">
         <x:v>106</x:v>
       </x:c>
-      <x:c r="AX215" t="s">
-        <x:v>1</x:v>
+      <x:c r="AX215" s="6" t="s">
+        <x:v>106</x:v>
       </x:c>
       <x:c r="AY215" s="6" t="s">
         <x:v>106</x:v>
@@ -58128,8 +58134,8 @@
       <x:c r="BA215" s="6" t="s">
         <x:v>106</x:v>
       </x:c>
-      <x:c r="BB215" t="s">
-        <x:v>1</x:v>
+      <x:c r="BB215" s="6" t="s">
+        <x:v>106</x:v>
       </x:c>
       <x:c r="BC215" s="6" t="s">
         <x:v>106</x:v>
@@ -58146,8 +58152,8 @@
       <x:c r="BG215" s="6" t="s">
         <x:v>106</x:v>
       </x:c>
-      <x:c r="BH215" s="6" t="s">
-        <x:v>106</x:v>
+      <x:c r="BH215" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="BI215" s="6" t="s">
         <x:v>106</x:v>
@@ -58158,8 +58164,8 @@
       <x:c r="BK215" s="6" t="s">
         <x:v>106</x:v>
       </x:c>
-      <x:c r="BL215" t="s">
-        <x:v>1</x:v>
+      <x:c r="BL215" s="6" t="s">
+        <x:v>106</x:v>
       </x:c>
       <x:c r="BM215" s="6" t="s">
         <x:v>106</x:v>
@@ -58170,8 +58176,8 @@
       <x:c r="BO215" s="6" t="s">
         <x:v>106</x:v>
       </x:c>
-      <x:c r="BP215" t="s">
-        <x:v>1</x:v>
+      <x:c r="BP215" s="6" t="s">
+        <x:v>106</x:v>
       </x:c>
       <x:c r="BQ215" t="s">
         <x:v>1</x:v>
@@ -58212,14 +58218,14 @@
       <x:c r="CC215" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CD215" s="6" t="s">
-        <x:v>106</x:v>
+      <x:c r="CD215" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="CE215" s="6" t="s">
         <x:v>106</x:v>
       </x:c>
-      <x:c r="CF215" t="s">
-        <x:v>1</x:v>
+      <x:c r="CF215" s="6" t="s">
+        <x:v>106</x:v>
       </x:c>
       <x:c r="CG215" s="6" t="s">
         <x:v>106</x:v>
@@ -58233,8 +58239,8 @@
       <x:c r="CJ215" s="6" t="s">
         <x:v>106</x:v>
       </x:c>
-      <x:c r="CK215" s="6" t="s">
-        <x:v>106</x:v>
+      <x:c r="CK215" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="CL215" s="6" t="s">
         <x:v>106</x:v>
@@ -58242,8 +58248,8 @@
       <x:c r="CM215" s="6" t="s">
         <x:v>106</x:v>
       </x:c>
-      <x:c r="CN215" t="s">
-        <x:v>1</x:v>
+      <x:c r="CN215" s="6" t="s">
+        <x:v>106</x:v>
       </x:c>
       <x:c r="CO215" s="6" t="s">
         <x:v>106</x:v>
@@ -58256,8 +58262,8 @@
       <x:c r="B216" s="5" t="s">
         <x:v>441</x:v>
       </x:c>
-      <x:c r="C216" t="s">
-        <x:v>1</x:v>
+      <x:c r="C216" s="6" t="s">
+        <x:v>106</x:v>
       </x:c>
       <x:c r="D216" t="s">
         <x:v>1</x:v>
@@ -58280,14 +58286,14 @@
       <x:c r="J216" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="K216" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="L216" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="M216" t="s">
-        <x:v>1</x:v>
+      <x:c r="K216" s="6" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="L216" s="6" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="M216" s="6" t="s">
+        <x:v>106</x:v>
       </x:c>
       <x:c r="N216" s="6" t="s">
         <x:v>106</x:v>
@@ -58298,35 +58304,35 @@
       <x:c r="P216" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="Q216" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="R216" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="S216" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="T216" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="U216" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="V216" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="W216" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="X216" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="Y216" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="Z216" t="s">
-        <x:v>1</x:v>
+      <x:c r="Q216" s="6" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="R216" s="6" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="S216" s="6" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="T216" s="6" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="U216" s="6" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="V216" s="6" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="W216" s="6" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="X216" s="6" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="Y216" s="6" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="Z216" s="6" t="s">
+        <x:v>106</x:v>
       </x:c>
       <x:c r="AA216" s="6" t="s">
         <x:v>106</x:v>
@@ -58361,8 +58367,8 @@
       <x:c r="AK216" s="6" t="s">
         <x:v>106</x:v>
       </x:c>
-      <x:c r="AL216" t="s">
-        <x:v>1</x:v>
+      <x:c r="AL216" s="6" t="s">
+        <x:v>106</x:v>
       </x:c>
       <x:c r="AM216" s="6" t="s">
         <x:v>106</x:v>
@@ -58382,8 +58388,8 @@
       <x:c r="AR216" s="6" t="s">
         <x:v>106</x:v>
       </x:c>
-      <x:c r="AS216" t="s">
-        <x:v>1</x:v>
+      <x:c r="AS216" s="6" t="s">
+        <x:v>106</x:v>
       </x:c>
       <x:c r="AT216" s="6" t="s">
         <x:v>106</x:v>
@@ -58397,8 +58403,8 @@
       <x:c r="AW216" s="6" t="s">
         <x:v>106</x:v>
       </x:c>
-      <x:c r="AX216" s="6" t="s">
-        <x:v>106</x:v>
+      <x:c r="AX216" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="AY216" s="6" t="s">
         <x:v>106</x:v>
@@ -58409,8 +58415,8 @@
       <x:c r="BA216" s="6" t="s">
         <x:v>106</x:v>
       </x:c>
-      <x:c r="BB216" s="6" t="s">
-        <x:v>106</x:v>
+      <x:c r="BB216" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="BC216" s="6" t="s">
         <x:v>106</x:v>
@@ -58427,8 +58433,8 @@
       <x:c r="BG216" s="6" t="s">
         <x:v>106</x:v>
       </x:c>
-      <x:c r="BH216" t="s">
-        <x:v>1</x:v>
+      <x:c r="BH216" s="6" t="s">
+        <x:v>106</x:v>
       </x:c>
       <x:c r="BI216" s="6" t="s">
         <x:v>106</x:v>
@@ -58439,8 +58445,8 @@
       <x:c r="BK216" s="6" t="s">
         <x:v>106</x:v>
       </x:c>
-      <x:c r="BL216" s="6" t="s">
-        <x:v>106</x:v>
+      <x:c r="BL216" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="BM216" s="6" t="s">
         <x:v>106</x:v>
@@ -58451,8 +58457,8 @@
       <x:c r="BO216" s="6" t="s">
         <x:v>106</x:v>
       </x:c>
-      <x:c r="BP216" s="6" t="s">
-        <x:v>106</x:v>
+      <x:c r="BP216" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="BQ216" t="s">
         <x:v>1</x:v>
@@ -58493,14 +58499,14 @@
       <x:c r="CC216" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CD216" t="s">
-        <x:v>1</x:v>
+      <x:c r="CD216" s="6" t="s">
+        <x:v>106</x:v>
       </x:c>
       <x:c r="CE216" s="6" t="s">
         <x:v>106</x:v>
       </x:c>
-      <x:c r="CF216" s="6" t="s">
-        <x:v>106</x:v>
+      <x:c r="CF216" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="CG216" s="6" t="s">
         <x:v>106</x:v>
@@ -58514,8 +58520,8 @@
       <x:c r="CJ216" s="6" t="s">
         <x:v>106</x:v>
       </x:c>
-      <x:c r="CK216" t="s">
-        <x:v>1</x:v>
+      <x:c r="CK216" s="6" t="s">
+        <x:v>106</x:v>
       </x:c>
       <x:c r="CL216" s="6" t="s">
         <x:v>106</x:v>
@@ -58523,8 +58529,8 @@
       <x:c r="CM216" s="6" t="s">
         <x:v>106</x:v>
       </x:c>
-      <x:c r="CN216" s="6" t="s">
-        <x:v>106</x:v>
+      <x:c r="CN216" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="CO216" s="6" t="s">
         <x:v>106</x:v>
@@ -58561,26 +58567,26 @@
       <x:c r="J217" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="K217" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="L217" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="M217" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="N217" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="O217" t="s">
-        <x:v>1</x:v>
+      <x:c r="K217" s="6" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="L217" s="6" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="M217" s="6" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="N217" s="6" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="O217" s="6" t="s">
+        <x:v>106</x:v>
       </x:c>
       <x:c r="P217" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="Q217" t="s">
-        <x:v>1</x:v>
+      <x:c r="Q217" s="6" t="s">
+        <x:v>106</x:v>
       </x:c>
       <x:c r="R217" t="s">
         <x:v>1</x:v>
@@ -58609,59 +58615,59 @@
       <x:c r="Z217" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="AA217" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AB217" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AC217" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AD217" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AE217" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AF217" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AG217" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AH217" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AI217" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AJ217" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AK217" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AL217" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AM217" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AN217" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AO217" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AP217" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AQ217" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AR217" t="s">
-        <x:v>1</x:v>
+      <x:c r="AA217" s="6" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="AB217" s="6" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="AC217" s="6" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="AD217" s="6" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="AE217" s="6" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="AF217" s="6" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="AG217" s="6" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="AH217" s="6" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="AI217" s="6" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="AJ217" s="6" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="AK217" s="6" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="AL217" s="6" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="AM217" s="6" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="AN217" s="6" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="AO217" s="6" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="AP217" s="6" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="AQ217" s="6" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="AR217" s="6" t="s">
+        <x:v>106</x:v>
       </x:c>
       <x:c r="AS217" t="s">
         <x:v>1</x:v>
@@ -58669,50 +58675,50 @@
       <x:c r="AT217" s="6" t="s">
         <x:v>106</x:v>
       </x:c>
-      <x:c r="AU217" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AV217" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AW217" t="s">
-        <x:v>1</x:v>
+      <x:c r="AU217" s="6" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="AV217" s="6" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="AW217" s="6" t="s">
+        <x:v>106</x:v>
       </x:c>
       <x:c r="AX217" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="AY217" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AZ217" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BA217" t="s">
-        <x:v>1</x:v>
+      <x:c r="AY217" s="6" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="AZ217" s="6" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="BA217" s="6" t="s">
+        <x:v>106</x:v>
       </x:c>
       <x:c r="BB217" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BC217" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BD217" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BE217" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BF217" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BG217" t="s">
-        <x:v>1</x:v>
+      <x:c r="BC217" s="6" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="BD217" s="6" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="BE217" s="6" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="BF217" s="6" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="BG217" s="6" t="s">
+        <x:v>106</x:v>
       </x:c>
       <x:c r="BH217" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BI217" t="s">
-        <x:v>1</x:v>
+      <x:c r="BI217" s="6" t="s">
+        <x:v>106</x:v>
       </x:c>
       <x:c r="BJ217" s="6" t="s">
         <x:v>106</x:v>
@@ -58723,14 +58729,14 @@
       <x:c r="BL217" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BM217" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BN217" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BO217" t="s">
-        <x:v>1</x:v>
+      <x:c r="BM217" s="6" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="BN217" s="6" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="BO217" s="6" t="s">
+        <x:v>106</x:v>
       </x:c>
       <x:c r="BP217" t="s">
         <x:v>1</x:v>
@@ -58741,11 +58747,11 @@
       <x:c r="BR217" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BS217" s="6" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="BT217" s="6" t="s">
-        <x:v>106</x:v>
+      <x:c r="BS217" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BT217" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="BU217" t="s">
         <x:v>1</x:v>
@@ -58753,11 +58759,11 @@
       <x:c r="BV217" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BW217" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BX217" t="s">
-        <x:v>1</x:v>
+      <x:c r="BW217" s="6" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="BX217" s="6" t="s">
+        <x:v>106</x:v>
       </x:c>
       <x:c r="BY217" t="s">
         <x:v>1</x:v>
@@ -58777,38 +58783,38 @@
       <x:c r="CD217" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CE217" t="s">
-        <x:v>1</x:v>
+      <x:c r="CE217" s="6" t="s">
+        <x:v>106</x:v>
       </x:c>
       <x:c r="CF217" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CG217" t="s">
-        <x:v>1</x:v>
+      <x:c r="CG217" s="6" t="s">
+        <x:v>106</x:v>
       </x:c>
       <x:c r="CH217" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CI217" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CJ217" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CK217" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CL217" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CM217" t="s">
-        <x:v>1</x:v>
+      <x:c r="CI217" s="6" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="CJ217" s="6" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="CK217" s="6" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="CL217" s="6" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="CM217" s="6" t="s">
+        <x:v>106</x:v>
       </x:c>
       <x:c r="CN217" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CO217" t="s">
-        <x:v>1</x:v>
+      <x:c r="CO217" s="6" t="s">
+        <x:v>106</x:v>
       </x:c>
     </x:row>
     <x:row r="218">
@@ -58848,20 +58854,20 @@
       <x:c r="L218" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="M218" s="6" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="N218" s="6" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="O218" s="6" t="s">
-        <x:v>106</x:v>
+      <x:c r="M218" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N218" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="O218" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="P218" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="Q218" s="6" t="s">
-        <x:v>106</x:v>
+      <x:c r="Q218" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="R218" t="s">
         <x:v>1</x:v>
@@ -58935,11 +58941,11 @@
       <x:c r="AO218" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="AP218" s="6" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="AQ218" s="6" t="s">
-        <x:v>106</x:v>
+      <x:c r="AP218" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AQ218" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="AR218" t="s">
         <x:v>1</x:v>
@@ -58947,50 +58953,50 @@
       <x:c r="AS218" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="AT218" s="6" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="AU218" s="6" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="AV218" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AW218" s="6" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="AX218" s="6" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="AY218" s="6" t="s">
-        <x:v>106</x:v>
+      <x:c r="AT218" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AU218" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AV218" s="6" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="AW218" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AX218" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AY218" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="AZ218" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BA218" s="6" t="s">
-        <x:v>106</x:v>
+      <x:c r="BA218" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="BB218" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BC218" s="6" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="BD218" s="6" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="BE218" s="6" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="BF218" s="6" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="BG218" s="6" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="BH218" s="6" t="s">
-        <x:v>106</x:v>
+      <x:c r="BC218" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BD218" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BE218" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BF218" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BG218" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BH218" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="BI218" t="s">
         <x:v>1</x:v>
@@ -59001,47 +59007,47 @@
       <x:c r="BK218" s="6" t="s">
         <x:v>106</x:v>
       </x:c>
-      <x:c r="BL218" s="6" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="BM218" s="6" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="BN218" s="6" t="s">
-        <x:v>106</x:v>
+      <x:c r="BL218" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BM218" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BN218" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="BO218" s="6" t="s">
         <x:v>106</x:v>
       </x:c>
-      <x:c r="BP218" s="6" t="s">
-        <x:v>106</x:v>
+      <x:c r="BP218" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="BQ218" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BR218" s="6" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="BS218" s="6" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="BT218" s="6" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="BU218" s="6" t="s">
-        <x:v>106</x:v>
+      <x:c r="BR218" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BS218" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BT218" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BU218" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="BV218" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BW218" s="6" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="BX218" s="6" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="BY218" s="6" t="s">
-        <x:v>106</x:v>
+      <x:c r="BW218" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BX218" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BY218" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="BZ218" t="s">
         <x:v>1</x:v>
@@ -59049,32 +59055,32 @@
       <x:c r="CA218" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CB218" s="6" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="CC218" s="6" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="CD218" s="6" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="CE218" s="6" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="CF218" s="6" t="s">
-        <x:v>106</x:v>
+      <x:c r="CB218" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CC218" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CD218" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CE218" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CF218" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="CG218" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CH218" s="6" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="CI218" s="6" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="CJ218" s="6" t="s">
-        <x:v>106</x:v>
+      <x:c r="CH218" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CI218" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CJ218" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="CK218" t="s">
         <x:v>1</x:v>
@@ -59085,11 +59091,11 @@
       <x:c r="CM218" s="6" t="s">
         <x:v>106</x:v>
       </x:c>
-      <x:c r="CN218" s="6" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="CO218" s="6" t="s">
-        <x:v>106</x:v>
+      <x:c r="CN218" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CO218" t="s">
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="219">
@@ -59102,32 +59108,32 @@
       <x:c r="C219" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D219" s="6" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="E219" s="6" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="F219" s="6" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="G219" s="6" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="H219" s="6" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="I219" s="6" t="s">
-        <x:v>106</x:v>
+      <x:c r="D219" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E219" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F219" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G219" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H219" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I219" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J219" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="K219" s="6" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="L219" s="6" t="s">
-        <x:v>106</x:v>
+      <x:c r="K219" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L219" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="M219" t="s">
         <x:v>1</x:v>
@@ -59138,38 +59144,38 @@
       <x:c r="O219" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="P219" s="6" t="s">
-        <x:v>106</x:v>
+      <x:c r="P219" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="Q219" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="R219" s="6" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="S219" s="6" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="T219" s="6" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="U219" s="6" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="V219" s="6" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="W219" s="6" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="X219" s="6" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="Y219" s="6" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="Z219" s="6" t="s">
-        <x:v>106</x:v>
+      <x:c r="R219" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="S219" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="T219" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U219" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="V219" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="W219" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="X219" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Y219" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Z219" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="AA219" t="s">
         <x:v>1</x:v>
@@ -59228,8 +59234,8 @@
       <x:c r="AS219" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="AT219" t="s">
-        <x:v>1</x:v>
+      <x:c r="AT219" s="6" t="s">
+        <x:v>106</x:v>
       </x:c>
       <x:c r="AU219" t="s">
         <x:v>1</x:v>
@@ -59276,11 +59282,11 @@
       <x:c r="BI219" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BJ219" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BK219" t="s">
-        <x:v>1</x:v>
+      <x:c r="BJ219" s="6" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="BK219" s="6" t="s">
+        <x:v>106</x:v>
       </x:c>
       <x:c r="BL219" t="s">
         <x:v>1</x:v>
@@ -59303,11 +59309,11 @@
       <x:c r="BR219" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BS219" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BT219" t="s">
-        <x:v>1</x:v>
+      <x:c r="BS219" s="6" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="BT219" s="6" t="s">
+        <x:v>106</x:v>
       </x:c>
       <x:c r="BU219" t="s">
         <x:v>1</x:v>
@@ -59327,8 +59333,8 @@
       <x:c r="BZ219" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CA219" s="6" t="s">
-        <x:v>106</x:v>
+      <x:c r="CA219" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="CB219" t="s">
         <x:v>1</x:v>
@@ -59404,11 +59410,11 @@
       <x:c r="J220" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="K220" s="6" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="L220" s="6" t="s">
-        <x:v>106</x:v>
+      <x:c r="K220" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L220" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="M220" s="6" t="s">
         <x:v>106</x:v>
@@ -59485,17 +59491,17 @@
       <x:c r="AK220" s="6" t="s">
         <x:v>106</x:v>
       </x:c>
-      <x:c r="AL220" s="6" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="AM220" s="6" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="AN220" s="6" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="AO220" s="6" t="s">
-        <x:v>106</x:v>
+      <x:c r="AL220" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AM220" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AN220" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AO220" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="AP220" s="6" t="s">
         <x:v>106</x:v>
@@ -59503,8 +59509,8 @@
       <x:c r="AQ220" s="6" t="s">
         <x:v>106</x:v>
       </x:c>
-      <x:c r="AR220" s="6" t="s">
-        <x:v>106</x:v>
+      <x:c r="AR220" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="AS220" t="s">
         <x:v>1</x:v>
@@ -59515,20 +59521,20 @@
       <x:c r="AU220" s="6" t="s">
         <x:v>106</x:v>
       </x:c>
-      <x:c r="AV220" s="6" t="s">
-        <x:v>106</x:v>
+      <x:c r="AV220" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="AW220" s="6" t="s">
         <x:v>106</x:v>
       </x:c>
-      <x:c r="AX220" t="s">
-        <x:v>1</x:v>
+      <x:c r="AX220" s="6" t="s">
+        <x:v>106</x:v>
       </x:c>
       <x:c r="AY220" s="6" t="s">
         <x:v>106</x:v>
       </x:c>
-      <x:c r="AZ220" s="6" t="s">
-        <x:v>106</x:v>
+      <x:c r="AZ220" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="BA220" s="6" t="s">
         <x:v>106</x:v>
@@ -59551,11 +59557,11 @@
       <x:c r="BG220" s="6" t="s">
         <x:v>106</x:v>
       </x:c>
-      <x:c r="BH220" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BI220" s="6" t="s">
-        <x:v>106</x:v>
+      <x:c r="BH220" s="6" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="BI220" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="BJ220" s="6" t="s">
         <x:v>106</x:v>
@@ -59563,8 +59569,8 @@
       <x:c r="BK220" s="6" t="s">
         <x:v>106</x:v>
       </x:c>
-      <x:c r="BL220" t="s">
-        <x:v>1</x:v>
+      <x:c r="BL220" s="6" t="s">
+        <x:v>106</x:v>
       </x:c>
       <x:c r="BM220" s="6" t="s">
         <x:v>106</x:v>
@@ -59575,23 +59581,23 @@
       <x:c r="BO220" s="6" t="s">
         <x:v>106</x:v>
       </x:c>
-      <x:c r="BP220" t="s">
-        <x:v>1</x:v>
+      <x:c r="BP220" s="6" t="s">
+        <x:v>106</x:v>
       </x:c>
       <x:c r="BQ220" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BR220" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BS220" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BT220" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BU220" t="s">
-        <x:v>1</x:v>
+      <x:c r="BR220" s="6" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="BS220" s="6" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="BT220" s="6" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="BU220" s="6" t="s">
+        <x:v>106</x:v>
       </x:c>
       <x:c r="BV220" t="s">
         <x:v>1</x:v>
@@ -59602,8 +59608,8 @@
       <x:c r="BX220" s="6" t="s">
         <x:v>106</x:v>
       </x:c>
-      <x:c r="BY220" t="s">
-        <x:v>1</x:v>
+      <x:c r="BY220" s="6" t="s">
+        <x:v>106</x:v>
       </x:c>
       <x:c r="BZ220" t="s">
         <x:v>1</x:v>
@@ -59611,26 +59617,26 @@
       <x:c r="CA220" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CB220" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CC220" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CD220" t="s">
-        <x:v>1</x:v>
+      <x:c r="CB220" s="6" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="CC220" s="6" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="CD220" s="6" t="s">
+        <x:v>106</x:v>
       </x:c>
       <x:c r="CE220" s="6" t="s">
         <x:v>106</x:v>
       </x:c>
-      <x:c r="CF220" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CG220" s="6" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="CH220" t="s">
-        <x:v>1</x:v>
+      <x:c r="CF220" s="6" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="CG220" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CH220" s="6" t="s">
+        <x:v>106</x:v>
       </x:c>
       <x:c r="CI220" s="6" t="s">
         <x:v>106</x:v>
@@ -59638,306 +59644,306 @@
       <x:c r="CJ220" s="6" t="s">
         <x:v>106</x:v>
       </x:c>
-      <x:c r="CK220" s="6" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="CL220" s="6" t="s">
-        <x:v>106</x:v>
+      <x:c r="CK220" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CL220" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="CM220" s="6" t="s">
         <x:v>106</x:v>
       </x:c>
-      <x:c r="CN220" t="s">
-        <x:v>1</x:v>
+      <x:c r="CN220" s="6" t="s">
+        <x:v>106</x:v>
       </x:c>
       <x:c r="CO220" s="6" t="s">
         <x:v>106</x:v>
       </x:c>
     </x:row>
     <x:row r="221">
-      <x:c r="A221" s="3" t="s">
+      <x:c r="A221" s="4" t="s">
         <x:v>450</x:v>
+      </x:c>
+      <x:c r="B221" s="5" t="s">
+        <x:v>451</x:v>
+      </x:c>
+      <x:c r="C221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D221" s="6" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="E221" s="6" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="F221" s="6" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="G221" s="6" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="H221" s="6" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="I221" s="6" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="J221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K221" s="6" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="L221" s="6" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="M221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="O221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P221" s="6" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="Q221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="R221" s="6" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="S221" s="6" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="T221" s="6" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="U221" s="6" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="V221" s="6" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="W221" s="6" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="X221" s="6" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="Y221" s="6" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="Z221" s="6" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="AA221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AB221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AC221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AD221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AE221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AF221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AG221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AH221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AI221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AJ221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AK221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AL221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AM221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AN221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AO221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AP221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AQ221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AR221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AS221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AT221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AU221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AV221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AW221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AX221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AY221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AZ221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BA221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BB221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BC221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BD221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BE221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BF221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BG221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BH221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BI221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BJ221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BK221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BL221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BM221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BN221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BO221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BP221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BQ221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BR221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BS221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BT221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BU221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BV221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BW221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BX221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BY221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BZ221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CA221" s="6" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="CB221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CC221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CD221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CE221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CF221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CG221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CH221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CI221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CJ221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CK221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CL221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CM221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CN221" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="CO221" t="s">
         <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="222">
-      <x:c r="A222" s="4" t="s">
-        <x:v>451</x:v>
-      </x:c>
-      <x:c r="B222" s="5" t="s">
+      <x:c r="A222" s="3" t="s">
         <x:v>452</x:v>
-      </x:c>
-      <x:c r="C222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="H222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="J222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="K222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="L222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="M222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="N222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="O222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="P222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="Q222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="R222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="S222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="T222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="U222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="V222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="W222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="X222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="Y222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="Z222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AA222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AB222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AC222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AD222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AE222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AF222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AG222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AH222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AI222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AJ222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AK222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AL222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AM222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AN222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AO222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AP222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AQ222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AR222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AS222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AT222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AU222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AV222" s="6" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="AW222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AX222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AY222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AZ222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BA222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BB222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BC222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BD222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BE222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BF222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BG222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BH222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BI222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BJ222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BK222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BL222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BM222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BN222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BO222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BP222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BQ222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BR222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BS222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BT222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BU222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BV222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BW222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BX222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BY222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BZ222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CA222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CB222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CC222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CD222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CE222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CF222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CG222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CH222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CI222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CJ222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CK222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CL222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CM222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CN222" t="s">
-        <x:v>1</x:v>
       </x:c>
       <x:c r="CO222" t="s">
         <x:v>1</x:v>
@@ -60085,8 +60091,8 @@
       <x:c r="AU223" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="AV223" t="s">
-        <x:v>1</x:v>
+      <x:c r="AV223" s="6" t="s">
+        <x:v>106</x:v>
       </x:c>
       <x:c r="AW223" t="s">
         <x:v>1</x:v>
@@ -60270,8 +60276,8 @@
       <x:c r="O224" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="P224" s="6" t="s">
-        <x:v>106</x:v>
+      <x:c r="P224" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="Q224" t="s">
         <x:v>1</x:v>
@@ -60510,7 +60516,7 @@
         <x:v>457</x:v>
       </x:c>
       <x:c r="B225" s="5" t="s">
-        <x:v>119</x:v>
+        <x:v>458</x:v>
       </x:c>
       <x:c r="C225" t="s">
         <x:v>1</x:v>
@@ -60551,8 +60557,8 @@
       <x:c r="O225" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="P225" t="s">
-        <x:v>1</x:v>
+      <x:c r="P225" s="6" t="s">
+        <x:v>106</x:v>
       </x:c>
       <x:c r="Q225" t="s">
         <x:v>1</x:v>
@@ -60713,8 +60719,8 @@
       <x:c r="BQ225" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BR225" s="6" t="s">
-        <x:v>106</x:v>
+      <x:c r="BR225" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="BS225" t="s">
         <x:v>1</x:v>
@@ -60788,10 +60794,10 @@
     </x:row>
     <x:row r="226">
       <x:c r="A226" s="4" t="s">
-        <x:v>458</x:v>
+        <x:v>459</x:v>
       </x:c>
       <x:c r="B226" s="5" t="s">
-        <x:v>459</x:v>
+        <x:v>119</x:v>
       </x:c>
       <x:c r="C226" t="s">
         <x:v>1</x:v>
@@ -60943,8 +60949,8 @@
       <x:c r="AZ226" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BA226" s="6" t="s">
-        <x:v>106</x:v>
+      <x:c r="BA226" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="BB226" t="s">
         <x:v>1</x:v>
@@ -60994,8 +61000,8 @@
       <x:c r="BQ226" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BR226" t="s">
-        <x:v>1</x:v>
+      <x:c r="BR226" s="6" t="s">
+        <x:v>106</x:v>
       </x:c>
       <x:c r="BS226" t="s">
         <x:v>1</x:v>
@@ -61030,8 +61036,8 @@
       <x:c r="CC226" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CD226" s="6" t="s">
-        <x:v>106</x:v>
+      <x:c r="CD226" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="CE226" t="s">
         <x:v>1</x:v>
@@ -61631,13 +61637,13 @@
     </x:row>
     <x:row r="229">
       <x:c r="A229" s="4" t="s">
-        <x:v>1</x:v>
+        <x:v>464</x:v>
       </x:c>
       <x:c r="B229" s="5" t="s">
-        <x:v>464</x:v>
-      </x:c>
-      <x:c r="C229" s="6" t="s">
-        <x:v>106</x:v>
+        <x:v>465</x:v>
+      </x:c>
+      <x:c r="C229" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D229" t="s">
         <x:v>1</x:v>
@@ -61681,11 +61687,11 @@
       <x:c r="Q229" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="R229" s="6" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="S229" s="6" t="s">
-        <x:v>106</x:v>
+      <x:c r="R229" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="S229" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="T229" t="s">
         <x:v>1</x:v>
@@ -61705,11 +61711,11 @@
       <x:c r="Y229" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="Z229" s="6" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="AA229" s="6" t="s">
-        <x:v>106</x:v>
+      <x:c r="Z229" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AA229" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="AB229" t="s">
         <x:v>1</x:v>
@@ -61726,20 +61732,20 @@
       <x:c r="AF229" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="AG229" s="6" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="AH229" s="6" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="AI229" s="6" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="AJ229" s="6" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="AK229" s="6" t="s">
-        <x:v>106</x:v>
+      <x:c r="AG229" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AH229" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AI229" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AJ229" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AK229" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="AL229" t="s">
         <x:v>1</x:v>
@@ -61786,8 +61792,8 @@
       <x:c r="AZ229" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BA229" t="s">
-        <x:v>1</x:v>
+      <x:c r="BA229" s="6" t="s">
+        <x:v>106</x:v>
       </x:c>
       <x:c r="BB229" t="s">
         <x:v>1</x:v>
@@ -61813,11 +61819,11 @@
       <x:c r="BI229" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BJ229" s="6" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="BK229" s="6" t="s">
-        <x:v>106</x:v>
+      <x:c r="BJ229" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BK229" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="BL229" t="s">
         <x:v>1</x:v>
@@ -61873,8 +61879,8 @@
       <x:c r="CC229" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CD229" t="s">
-        <x:v>1</x:v>
+      <x:c r="CD229" s="6" t="s">
+        <x:v>106</x:v>
       </x:c>
       <x:c r="CE229" t="s">
         <x:v>1</x:v>
@@ -61915,10 +61921,10 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="B230" s="5" t="s">
-        <x:v>465</x:v>
-      </x:c>
-      <x:c r="C230" t="s">
-        <x:v>1</x:v>
+        <x:v>466</x:v>
+      </x:c>
+      <x:c r="C230" s="6" t="s">
+        <x:v>106</x:v>
       </x:c>
       <x:c r="D230" t="s">
         <x:v>1</x:v>
@@ -61962,11 +61968,11 @@
       <x:c r="Q230" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="R230" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="S230" t="s">
-        <x:v>1</x:v>
+      <x:c r="R230" s="6" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="S230" s="6" t="s">
+        <x:v>106</x:v>
       </x:c>
       <x:c r="T230" t="s">
         <x:v>1</x:v>
@@ -61986,11 +61992,11 @@
       <x:c r="Y230" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="Z230" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AA230" t="s">
-        <x:v>1</x:v>
+      <x:c r="Z230" s="6" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="AA230" s="6" t="s">
+        <x:v>106</x:v>
       </x:c>
       <x:c r="AB230" t="s">
         <x:v>1</x:v>
@@ -62007,20 +62013,20 @@
       <x:c r="AF230" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="AG230" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AH230" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AI230" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AJ230" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AK230" t="s">
-        <x:v>1</x:v>
+      <x:c r="AG230" s="6" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="AH230" s="6" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="AI230" s="6" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="AJ230" s="6" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="AK230" s="6" t="s">
+        <x:v>106</x:v>
       </x:c>
       <x:c r="AL230" t="s">
         <x:v>1</x:v>
@@ -62070,8 +62076,8 @@
       <x:c r="BA230" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BB230" s="6" t="s">
-        <x:v>106</x:v>
+      <x:c r="BB230" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="BC230" t="s">
         <x:v>1</x:v>
@@ -62094,11 +62100,11 @@
       <x:c r="BI230" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BJ230" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BK230" t="s">
-        <x:v>1</x:v>
+      <x:c r="BJ230" s="6" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="BK230" s="6" t="s">
+        <x:v>106</x:v>
       </x:c>
       <x:c r="BL230" t="s">
         <x:v>1</x:v>
@@ -62192,283 +62198,564 @@
       </x:c>
     </x:row>
     <x:row r="231">
-      <x:c r="A231" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="B231" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C231" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D231" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E231" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F231" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G231" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="H231" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I231" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="J231" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="K231" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="L231" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="M231" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="N231" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="O231" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="P231" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="Q231" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="R231" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="S231" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="T231" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="U231" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="V231" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="W231" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="X231" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="Y231" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="Z231" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AA231" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AB231" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AC231" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AD231" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AE231" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AF231" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AG231" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AH231" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AI231" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AJ231" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AK231" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AL231" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AM231" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AN231" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AO231" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AP231" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AQ231" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AR231" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AS231" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AT231" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AU231" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AV231" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AW231" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AX231" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AY231" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AZ231" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BA231" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BB231" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BC231" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BD231" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BE231" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BF231" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BG231" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BH231" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BI231" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BJ231" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BK231" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BL231" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BM231" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BN231" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BO231" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BP231" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BQ231" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BR231" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BS231" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BT231" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BU231" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BV231" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BW231" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BX231" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BY231" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BZ231" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CA231" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CB231" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CC231" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CD231" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CE231" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CF231" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CG231" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CH231" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CI231" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CJ231" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CK231" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CL231" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CM231" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CN231" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CO231" s="7" t="s">
+      <x:c r="A231" s="4" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B231" s="5" t="s">
+        <x:v>467</x:v>
+      </x:c>
+      <x:c r="C231" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D231" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E231" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F231" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G231" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H231" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I231" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J231" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K231" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L231" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M231" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N231" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="O231" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P231" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Q231" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="R231" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="S231" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="T231" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U231" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="V231" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="W231" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="X231" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Y231" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Z231" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AA231" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AB231" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AC231" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AD231" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AE231" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AF231" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AG231" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AH231" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AI231" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AJ231" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AK231" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AL231" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AM231" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AN231" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AO231" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AP231" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AQ231" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AR231" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AS231" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AT231" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AU231" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AV231" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AW231" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AX231" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AY231" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AZ231" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BA231" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BB231" s="6" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="BC231" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BD231" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BE231" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BF231" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BG231" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BH231" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BI231" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BJ231" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BK231" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BL231" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BM231" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BN231" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BO231" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BP231" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BQ231" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BR231" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BS231" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BT231" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BU231" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BV231" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BW231" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BX231" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BY231" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BZ231" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CA231" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CB231" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CC231" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CD231" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CE231" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CF231" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CG231" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CH231" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CI231" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CJ231" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CK231" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CL231" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CM231" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CN231" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CO231" t="s">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="232">
+      <x:c r="A232" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B232" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C232" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D232" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E232" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F232" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G232" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H232" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I232" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J232" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K232" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L232" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M232" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N232" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="O232" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P232" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Q232" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="R232" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="S232" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="T232" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U232" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="V232" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="W232" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="X232" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Y232" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Z232" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AA232" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AB232" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AC232" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AD232" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AE232" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AF232" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AG232" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AH232" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AI232" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AJ232" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AK232" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AL232" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AM232" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AN232" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AO232" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AP232" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AQ232" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AR232" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AS232" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AT232" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AU232" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AV232" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AW232" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AX232" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AY232" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AZ232" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BA232" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BB232" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BC232" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BD232" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BE232" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BF232" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BG232" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BH232" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BI232" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BJ232" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BK232" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BL232" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BM232" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BN232" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BO232" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BP232" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BQ232" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BR232" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BS232" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BT232" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BU232" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BV232" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BW232" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BX232" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BY232" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BZ232" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CA232" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CB232" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CC232" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CD232" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CE232" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CF232" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CG232" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CH232" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CI232" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CJ232" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CK232" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CL232" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CM232" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CN232" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CO232" s="7" t="s">
         <x:v>1</x:v>
       </x:c>
     </x:row>
@@ -62520,7 +62807,7 @@
     <x:mergeCell ref="A187:CO187"/>
     <x:mergeCell ref="A194:CO194"/>
     <x:mergeCell ref="A205:CO205"/>
-    <x:mergeCell ref="A221:CO221"/>
+    <x:mergeCell ref="A222:CO222"/>
   </x:mergeCells>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Update REAL engines (C++, Python, Rust): 2026.8.2.
</commit_message>
<xml_diff>
--- a/RegexFeatureMatrix.xlsx
+++ b/RegexFeatureMatrix.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="R0aaa27c948b64736"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="Rb7da85c239e2471c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -139,7 +139,7 @@
   </x:si>
   <x:si>
     <x:t>REAL
- 2026.7.63 </x:t>
+ 2026.8.2 </x:t>
   </x:si>
   <x:si>
     <x:t>ECMAScript</x:t>

</xml_diff>

<commit_message>
Update ICU engine: 78.3.
</commit_message>
<xml_diff>
--- a/RegexFeatureMatrix.xlsx
+++ b/RegexFeatureMatrix.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="Rb7da85c239e2471c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="Rfeecdc97b9a34188"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -67,7 +67,7 @@
   </x:si>
   <x:si>
     <x:t>ICU
- 77.1 </x:t>
+ 78.3 </x:t>
   </x:si>
   <x:si>
     <x:t>Rust

</xml_diff>

<commit_message>
Update 'regexp2' 2.6.0 and 'coregex' 0.12.23 (Go).
</commit_message>
<xml_diff>
--- a/RegexFeatureMatrix.xlsx
+++ b/RegexFeatureMatrix.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="R70f1fdd5a495426c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="R1fb02e5d43dd48c4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -7059,8 +7059,8 @@
       <x:c r="CG21" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CH21" t="s">
-        <x:v>1</x:v>
+      <x:c r="CH21" s="6" t="s">
+        <x:v>107</x:v>
       </x:c>
       <x:c r="CI21" t="s">
         <x:v>1</x:v>
@@ -7343,8 +7343,8 @@
       <x:c r="CG22" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CH22" t="s">
-        <x:v>1</x:v>
+      <x:c r="CH22" s="6" t="s">
+        <x:v>107</x:v>
       </x:c>
       <x:c r="CI22" t="s">
         <x:v>1</x:v>
@@ -10475,8 +10475,8 @@
       <x:c r="CG34" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CH34" t="s">
-        <x:v>1</x:v>
+      <x:c r="CH34" s="6" t="s">
+        <x:v>107</x:v>
       </x:c>
       <x:c r="CI34" t="s">
         <x:v>1</x:v>
@@ -26403,8 +26403,8 @@
       <x:c r="CG93" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CH93" t="s">
-        <x:v>1</x:v>
+      <x:c r="CH93" s="6" t="s">
+        <x:v>107</x:v>
       </x:c>
       <x:c r="CI93" t="s">
         <x:v>1</x:v>
@@ -28107,8 +28107,8 @@
       <x:c r="CG99" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CH99" t="s">
-        <x:v>1</x:v>
+      <x:c r="CH99" s="6" t="s">
+        <x:v>107</x:v>
       </x:c>
       <x:c r="CI99" t="s">
         <x:v>1</x:v>

</xml_diff>

<commit_message>
Update REAL engines (C++, Python, Rust): 2026.8.11. Update Feature Matrix for 'regexr'.
</commit_message>
<xml_diff>
--- a/RegexFeatureMatrix.xlsx
+++ b/RegexFeatureMatrix.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="R1fb02e5d43dd48c4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="R658cbb8358d84bce"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -139,7 +139,7 @@
   </x:si>
   <x:si>
     <x:t>REAL
- 2026.8.9 </x:t>
+ 2026.8.11 </x:t>
   </x:si>
   <x:si>
     <x:t>ECMAScript</x:t>
@@ -4700,8 +4700,8 @@
       <x:c r="BD13" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BE13" t="s">
-        <x:v>1</x:v>
+      <x:c r="BE13" s="6" t="s">
+        <x:v>107</x:v>
       </x:c>
       <x:c r="BF13" t="s">
         <x:v>1</x:v>
@@ -14372,8 +14372,8 @@
       <x:c r="BD49" s="6" t="s">
         <x:v>107</x:v>
       </x:c>
-      <x:c r="BE49" t="s">
-        <x:v>1</x:v>
+      <x:c r="BE49" s="6" t="s">
+        <x:v>107</x:v>
       </x:c>
       <x:c r="BF49" s="6" t="s">
         <x:v>107</x:v>
@@ -15792,8 +15792,8 @@
       <x:c r="BD54" s="6" t="s">
         <x:v>107</x:v>
       </x:c>
-      <x:c r="BE54" t="s">
-        <x:v>1</x:v>
+      <x:c r="BE54" s="6" t="s">
+        <x:v>107</x:v>
       </x:c>
       <x:c r="BF54" s="6" t="s">
         <x:v>107</x:v>
@@ -17504,8 +17504,8 @@
       <x:c r="BD61" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BE61" t="s">
-        <x:v>1</x:v>
+      <x:c r="BE61" s="6" t="s">
+        <x:v>107</x:v>
       </x:c>
       <x:c r="BF61" t="s">
         <x:v>1</x:v>
@@ -20912,8 +20912,8 @@
       <x:c r="BD73" s="6" t="s">
         <x:v>107</x:v>
       </x:c>
-      <x:c r="BE73" t="s">
-        <x:v>1</x:v>
+      <x:c r="BE73" s="6" t="s">
+        <x:v>107</x:v>
       </x:c>
       <x:c r="BF73" s="6" t="s">
         <x:v>107</x:v>
@@ -22332,8 +22332,8 @@
       <x:c r="BD78" s="6" t="s">
         <x:v>107</x:v>
       </x:c>
-      <x:c r="BE78" t="s">
-        <x:v>1</x:v>
+      <x:c r="BE78" s="6" t="s">
+        <x:v>107</x:v>
       </x:c>
       <x:c r="BF78" s="6" t="s">
         <x:v>107</x:v>
@@ -25180,8 +25180,8 @@
       <x:c r="BD89" s="6" t="s">
         <x:v>107</x:v>
       </x:c>
-      <x:c r="BE89" t="s">
-        <x:v>1</x:v>
+      <x:c r="BE89" s="6" t="s">
+        <x:v>107</x:v>
       </x:c>
       <x:c r="BF89" s="6" t="s">
         <x:v>107</x:v>
@@ -25748,8 +25748,8 @@
       <x:c r="BD91" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BE91" t="s">
-        <x:v>1</x:v>
+      <x:c r="BE91" s="6" t="s">
+        <x:v>107</x:v>
       </x:c>
       <x:c r="BF91" t="s">
         <x:v>1</x:v>
@@ -26316,8 +26316,8 @@
       <x:c r="BD93" s="6" t="s">
         <x:v>107</x:v>
       </x:c>
-      <x:c r="BE93" t="s">
-        <x:v>1</x:v>
+      <x:c r="BE93" s="6" t="s">
+        <x:v>107</x:v>
       </x:c>
       <x:c r="BF93" s="6" t="s">
         <x:v>107</x:v>
@@ -29448,8 +29448,8 @@
       <x:c r="BD105" s="6" t="s">
         <x:v>107</x:v>
       </x:c>
-      <x:c r="BE105" t="s">
-        <x:v>1</x:v>
+      <x:c r="BE105" s="6" t="s">
+        <x:v>107</x:v>
       </x:c>
       <x:c r="BF105" s="6" t="s">
         <x:v>107</x:v>
@@ -32572,8 +32572,8 @@
       <x:c r="BD116" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BE116" t="s">
-        <x:v>1</x:v>
+      <x:c r="BE116" s="6" t="s">
+        <x:v>107</x:v>
       </x:c>
       <x:c r="BF116" t="s">
         <x:v>1</x:v>
@@ -33432,8 +33432,8 @@
       <x:c r="BD120" s="6" t="s">
         <x:v>107</x:v>
       </x:c>
-      <x:c r="BE120" t="s">
-        <x:v>1</x:v>
+      <x:c r="BE120" s="6" t="s">
+        <x:v>107</x:v>
       </x:c>
       <x:c r="BF120" s="6" t="s">
         <x:v>107</x:v>
@@ -35704,8 +35704,8 @@
       <x:c r="BD128" s="6" t="s">
         <x:v>107</x:v>
       </x:c>
-      <x:c r="BE128" t="s">
-        <x:v>1</x:v>
+      <x:c r="BE128" s="6" t="s">
+        <x:v>107</x:v>
       </x:c>
       <x:c r="BF128" s="6" t="s">
         <x:v>107</x:v>
@@ -36272,8 +36272,8 @@
       <x:c r="BD130" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BE130" t="s">
-        <x:v>1</x:v>
+      <x:c r="BE130" s="6" t="s">
+        <x:v>107</x:v>
       </x:c>
       <x:c r="BF130" t="s">
         <x:v>1</x:v>
@@ -36556,8 +36556,8 @@
       <x:c r="BD131" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BE131" t="s">
-        <x:v>1</x:v>
+      <x:c r="BE131" s="6" t="s">
+        <x:v>107</x:v>
       </x:c>
       <x:c r="BF131" t="s">
         <x:v>1</x:v>
@@ -41400,8 +41400,8 @@
       <x:c r="BD150" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BE150" t="s">
-        <x:v>1</x:v>
+      <x:c r="BE150" s="6" t="s">
+        <x:v>107</x:v>
       </x:c>
       <x:c r="BF150" t="s">
         <x:v>1</x:v>
@@ -43388,8 +43388,8 @@
       <x:c r="BD157" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BE157" t="s">
-        <x:v>1</x:v>
+      <x:c r="BE157" s="6" t="s">
+        <x:v>107</x:v>
       </x:c>
       <x:c r="BF157" t="s">
         <x:v>1</x:v>
@@ -43672,8 +43672,8 @@
       <x:c r="BD158" s="6" t="s">
         <x:v>107</x:v>
       </x:c>
-      <x:c r="BE158" t="s">
-        <x:v>1</x:v>
+      <x:c r="BE158" s="6" t="s">
+        <x:v>107</x:v>
       </x:c>
       <x:c r="BF158" s="6" t="s">
         <x:v>107</x:v>
@@ -43956,8 +43956,8 @@
       <x:c r="BD159" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BE159" t="s">
-        <x:v>1</x:v>
+      <x:c r="BE159" s="6" t="s">
+        <x:v>107</x:v>
       </x:c>
       <x:c r="BF159" t="s">
         <x:v>1</x:v>
@@ -47648,8 +47648,8 @@
       <x:c r="BD172" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BE172" t="s">
-        <x:v>1</x:v>
+      <x:c r="BE172" s="6" t="s">
+        <x:v>107</x:v>
       </x:c>
       <x:c r="BF172" t="s">
         <x:v>1</x:v>
@@ -58472,8 +58472,8 @@
       <x:c r="BD214" s="6" t="s">
         <x:v>107</x:v>
       </x:c>
-      <x:c r="BE214" t="s">
-        <x:v>1</x:v>
+      <x:c r="BE214" s="6" t="s">
+        <x:v>107</x:v>
       </x:c>
       <x:c r="BF214" s="6" t="s">
         <x:v>107</x:v>
@@ -58756,8 +58756,8 @@
       <x:c r="BD215" s="6" t="s">
         <x:v>107</x:v>
       </x:c>
-      <x:c r="BE215" t="s">
-        <x:v>1</x:v>
+      <x:c r="BE215" s="6" t="s">
+        <x:v>107</x:v>
       </x:c>
       <x:c r="BF215" s="6" t="s">
         <x:v>107</x:v>
@@ -59040,8 +59040,8 @@
       <x:c r="BD216" s="6" t="s">
         <x:v>107</x:v>
       </x:c>
-      <x:c r="BE216" t="s">
-        <x:v>1</x:v>
+      <x:c r="BE216" s="6" t="s">
+        <x:v>107</x:v>
       </x:c>
       <x:c r="BF216" s="6" t="s">
         <x:v>107</x:v>
@@ -59324,8 +59324,8 @@
       <x:c r="BD217" s="6" t="s">
         <x:v>107</x:v>
       </x:c>
-      <x:c r="BE217" t="s">
-        <x:v>1</x:v>
+      <x:c r="BE217" s="6" t="s">
+        <x:v>107</x:v>
       </x:c>
       <x:c r="BF217" s="6" t="s">
         <x:v>107</x:v>

</xml_diff>

<commit_message>
Update REAL engines (C++, Python, Rust): 2026.8.14.
</commit_message>
<xml_diff>
--- a/RegexFeatureMatrix.xlsx
+++ b/RegexFeatureMatrix.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="R658cbb8358d84bce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="R864bd3a6973d424a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -139,7 +139,7 @@
   </x:si>
   <x:si>
     <x:t>REAL
- 2026.8.11 </x:t>
+ 2026.8.14 </x:t>
   </x:si>
   <x:si>
     <x:t>ECMAScript</x:t>

</xml_diff>

<commit_message>
Update REAL engines (C++, Python, Rust): 2026.8.16.
</commit_message>
<xml_diff>
--- a/RegexFeatureMatrix.xlsx
+++ b/RegexFeatureMatrix.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="R864bd3a6973d424a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="Ra5deac12fd9a4d6a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -139,7 +139,7 @@
   </x:si>
   <x:si>
     <x:t>REAL
- 2026.8.14 </x:t>
+ 2026.8.16 </x:t>
   </x:si>
   <x:si>
     <x:t>ECMAScript</x:t>

</xml_diff>

<commit_message>
Update REAL engines (C++, Python, Rust): 2026.8.19.
</commit_message>
<xml_diff>
--- a/RegexFeatureMatrix.xlsx
+++ b/RegexFeatureMatrix.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="R74aae3860d32421d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="Reb2729751cd94b1c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -135,7 +135,7 @@
   </x:si>
   <x:si>
     <x:t>REAL
- 2026.8.17 </x:t>
+ 2026.8.19 </x:t>
   </x:si>
   <x:si>
     <x:t>Regex</x:t>
@@ -15809,8 +15809,8 @@
       <x:c r="BE52" s="6" t="s">
         <x:v>112</x:v>
       </x:c>
-      <x:c r="BF52" t="s">
-        <x:v>1</x:v>
+      <x:c r="BF52" s="6" t="s">
+        <x:v>112</x:v>
       </x:c>
       <x:c r="BG52" t="s">
         <x:v>1</x:v>
@@ -15842,11 +15842,11 @@
       <x:c r="BP52" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BQ52" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BR52" t="s">
-        <x:v>1</x:v>
+      <x:c r="BQ52" s="6" t="s">
+        <x:v>112</x:v>
+      </x:c>
+      <x:c r="BR52" s="6" t="s">
+        <x:v>112</x:v>
       </x:c>
       <x:c r="BS52" t="s">
         <x:v>1</x:v>
@@ -15926,11 +15926,11 @@
       <x:c r="CR52" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CS52" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CT52" t="s">
-        <x:v>1</x:v>
+      <x:c r="CS52" s="6" t="s">
+        <x:v>112</x:v>
+      </x:c>
+      <x:c r="CT52" s="6" t="s">
+        <x:v>112</x:v>
       </x:c>
     </x:row>
     <x:row r="53">
@@ -22625,8 +22625,8 @@
       <x:c r="BE76" s="6" t="s">
         <x:v>112</x:v>
       </x:c>
-      <x:c r="BF76" t="s">
-        <x:v>1</x:v>
+      <x:c r="BF76" s="6" t="s">
+        <x:v>112</x:v>
       </x:c>
       <x:c r="BG76" t="s">
         <x:v>1</x:v>
@@ -22658,11 +22658,11 @@
       <x:c r="BP76" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BQ76" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BR76" t="s">
-        <x:v>1</x:v>
+      <x:c r="BQ76" s="6" t="s">
+        <x:v>112</x:v>
+      </x:c>
+      <x:c r="BR76" s="6" t="s">
+        <x:v>112</x:v>
       </x:c>
       <x:c r="BS76" t="s">
         <x:v>1</x:v>
@@ -22742,11 +22742,11 @@
       <x:c r="CR76" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CS76" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CT76" t="s">
-        <x:v>1</x:v>
+      <x:c r="CS76" s="6" t="s">
+        <x:v>112</x:v>
+      </x:c>
+      <x:c r="CT76" s="6" t="s">
+        <x:v>112</x:v>
       </x:c>
     </x:row>
     <x:row r="77">

</xml_diff>

<commit_message>
Update Lokad.Utf8Regex engine: 0.3.0.
</commit_message>
<xml_diff>
--- a/RegexFeatureMatrix.xlsx
+++ b/RegexFeatureMatrix.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="Reb2729751cd94b1c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="Rf1d7c01466074b3e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -5573,8 +5573,8 @@
       <x:c r="E16" s="6" t="s">
         <x:v>112</x:v>
       </x:c>
-      <x:c r="F16" s="6" t="s">
-        <x:v>112</x:v>
+      <x:c r="F16" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G16" t="s">
         <x:v>1</x:v>
@@ -43812,8 +43812,8 @@
       <x:c r="B153" s="5" t="s">
         <x:v>342</x:v>
       </x:c>
-      <x:c r="C153" t="s">
-        <x:v>1</x:v>
+      <x:c r="C153" s="6" t="s">
+        <x:v>112</x:v>
       </x:c>
       <x:c r="D153" t="s">
         <x:v>1</x:v>
@@ -43821,8 +43821,8 @@
       <x:c r="E153" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="F153" s="6" t="s">
-        <x:v>112</x:v>
+      <x:c r="F153" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G153" t="s">
         <x:v>1</x:v>

</xml_diff>

<commit_message>
Update engines to Rust 1.98.0. Update 'regress' 0.12.0 and 'resharp' 0.6.20.
</commit_message>
<xml_diff>
--- a/RegexFeatureMatrix.xlsx
+++ b/RegexFeatureMatrix.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="R8c7589d7656f4b2d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="R276e8a5dbaab4a2c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -71,7 +71,7 @@
   </x:si>
   <x:si>
     <x:t>Rust
- 1.97.1 </x:t>
+ 1.98.0 </x:t>
   </x:si>
   <x:si>
     <x:t>Java

</xml_diff>

<commit_message>
New experimental engine: 'Onigmo go-regexp' 0.1.3 (Go).
</commit_message>
<xml_diff>
--- a/RegexFeatureMatrix.xlsx
+++ b/RegexFeatureMatrix.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="Rbed83f87198e4a1c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="R957cdd86f644428a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -127,7 +127,7 @@
   </x:si>
   <x:si>
     <x:t>Go
- 1.26.5 </x:t>
+ 1.27.0 </x:t>
   </x:si>
   <x:si>
     <x:t>Dart
@@ -348,7 +348,7 @@
     <x:t>coregex</x:t>
   </x:si>
   <x:si>
-    <x:t>coregex (posix)</x:t>
+    <x:t>onigmo</x:t>
   </x:si>
   <x:si>
     <x:t>RegExp</x:t>
@@ -1685,7 +1685,7 @@
     <x:col min="90" max="90" width="8.498000000000001" customWidth="1"/>
     <x:col min="91" max="91" width="5.498" customWidth="1"/>
     <x:col min="92" max="92" width="8.398" customWidth="1"/>
-    <x:col min="93" max="93" width="14.292" customWidth="1"/>
+    <x:col min="93" max="93" width="7.897" customWidth="1"/>
     <x:col min="94" max="94" width="8.396" customWidth="1"/>
     <x:col min="95" max="95" width="16.391" customWidth="1"/>
     <x:col min="96" max="96" width="10.996" customWidth="1"/>
@@ -4650,8 +4650,8 @@
       <x:c r="CN12" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CO12" t="s">
-        <x:v>1</x:v>
+      <x:c r="CO12" s="6" t="s">
+        <x:v>112</x:v>
       </x:c>
       <x:c r="CP12" t="s">
         <x:v>1</x:v>
@@ -6722,8 +6722,8 @@
       <x:c r="CN19" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CO19" t="s">
-        <x:v>1</x:v>
+      <x:c r="CO19" s="6" t="s">
+        <x:v>112</x:v>
       </x:c>
       <x:c r="CP19" t="s">
         <x:v>1</x:v>
@@ -7314,8 +7314,8 @@
       <x:c r="CN21" s="6" t="s">
         <x:v>112</x:v>
       </x:c>
-      <x:c r="CO21" s="6" t="s">
-        <x:v>112</x:v>
+      <x:c r="CO21" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="CP21" t="s">
         <x:v>1</x:v>
@@ -10874,8 +10874,8 @@
       <x:c r="CN34" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CO34" t="s">
-        <x:v>1</x:v>
+      <x:c r="CO34" s="6" t="s">
+        <x:v>112</x:v>
       </x:c>
       <x:c r="CP34" t="s">
         <x:v>1</x:v>
@@ -11770,8 +11770,8 @@
       <x:c r="CN38" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CO38" t="s">
-        <x:v>1</x:v>
+      <x:c r="CO38" s="6" t="s">
+        <x:v>112</x:v>
       </x:c>
       <x:c r="CP38" t="s">
         <x:v>1</x:v>
@@ -13842,8 +13842,8 @@
       <x:c r="CN45" s="6" t="s">
         <x:v>112</x:v>
       </x:c>
-      <x:c r="CO45" s="6" t="s">
-        <x:v>112</x:v>
+      <x:c r="CO45" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="CP45" s="6" t="s">
         <x:v>112</x:v>
@@ -15026,8 +15026,8 @@
       <x:c r="CN49" s="6" t="s">
         <x:v>112</x:v>
       </x:c>
-      <x:c r="CO49" s="6" t="s">
-        <x:v>112</x:v>
+      <x:c r="CO49" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="CP49" t="s">
         <x:v>1</x:v>
@@ -18290,8 +18290,8 @@
       <x:c r="CN61" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CO61" t="s">
-        <x:v>1</x:v>
+      <x:c r="CO61" s="6" t="s">
+        <x:v>112</x:v>
       </x:c>
       <x:c r="CP61" s="6" t="s">
         <x:v>112</x:v>
@@ -18586,8 +18586,8 @@
       <x:c r="CN62" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CO62" t="s">
-        <x:v>1</x:v>
+      <x:c r="CO62" s="6" t="s">
+        <x:v>112</x:v>
       </x:c>
       <x:c r="CP62" t="s">
         <x:v>1</x:v>
@@ -20658,8 +20658,8 @@
       <x:c r="CN69" s="6" t="s">
         <x:v>112</x:v>
       </x:c>
-      <x:c r="CO69" s="6" t="s">
-        <x:v>112</x:v>
+      <x:c r="CO69" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="CP69" s="6" t="s">
         <x:v>112</x:v>
@@ -21842,8 +21842,8 @@
       <x:c r="CN73" s="6" t="s">
         <x:v>112</x:v>
       </x:c>
-      <x:c r="CO73" s="6" t="s">
-        <x:v>112</x:v>
+      <x:c r="CO73" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="CP73" t="s">
         <x:v>1</x:v>
@@ -25994,8 +25994,8 @@
       <x:c r="CN88" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CO88" t="s">
-        <x:v>1</x:v>
+      <x:c r="CO88" s="6" t="s">
+        <x:v>112</x:v>
       </x:c>
       <x:c r="CP88" t="s">
         <x:v>1</x:v>
@@ -27474,8 +27474,8 @@
       <x:c r="CN93" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CO93" t="s">
-        <x:v>1</x:v>
+      <x:c r="CO93" s="6" t="s">
+        <x:v>112</x:v>
       </x:c>
       <x:c r="CP93" t="s">
         <x:v>1</x:v>
@@ -29546,8 +29546,8 @@
       <x:c r="CN100" s="6" t="s">
         <x:v>112</x:v>
       </x:c>
-      <x:c r="CO100" s="6" t="s">
-        <x:v>112</x:v>
+      <x:c r="CO100" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="CP100" t="s">
         <x:v>1</x:v>
@@ -30442,8 +30442,8 @@
       <x:c r="CN104" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CO104" t="s">
-        <x:v>1</x:v>
+      <x:c r="CO104" s="6" t="s">
+        <x:v>112</x:v>
       </x:c>
       <x:c r="CP104" t="s">
         <x:v>1</x:v>
@@ -33402,8 +33402,8 @@
       <x:c r="CN114" s="6" t="s">
         <x:v>112</x:v>
       </x:c>
-      <x:c r="CO114" s="6" t="s">
-        <x:v>112</x:v>
+      <x:c r="CO114" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="CP114" t="s">
         <x:v>1</x:v>
@@ -39338,8 +39338,8 @@
       <x:c r="CN136" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CO136" t="s">
-        <x:v>1</x:v>
+      <x:c r="CO136" s="6" t="s">
+        <x:v>112</x:v>
       </x:c>
       <x:c r="CP136" t="s">
         <x:v>1</x:v>
@@ -40226,8 +40226,8 @@
       <x:c r="CN139" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CO139" t="s">
-        <x:v>1</x:v>
+      <x:c r="CO139" s="6" t="s">
+        <x:v>112</x:v>
       </x:c>
       <x:c r="CP139" t="s">
         <x:v>1</x:v>
@@ -43194,8 +43194,8 @@
       <x:c r="CN150" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CO150" t="s">
-        <x:v>1</x:v>
+      <x:c r="CO150" s="6" t="s">
+        <x:v>112</x:v>
       </x:c>
       <x:c r="CP150" t="s">
         <x:v>1</x:v>
@@ -43786,8 +43786,8 @@
       <x:c r="CN152" s="6" t="s">
         <x:v>112</x:v>
       </x:c>
-      <x:c r="CO152" s="6" t="s">
-        <x:v>112</x:v>
+      <x:c r="CO152" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="CP152" t="s">
         <x:v>1</x:v>
@@ -44378,8 +44378,8 @@
       <x:c r="CN154" s="6" t="s">
         <x:v>112</x:v>
       </x:c>
-      <x:c r="CO154" s="6" t="s">
-        <x:v>112</x:v>
+      <x:c r="CO154" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="CP154" s="6" t="s">
         <x:v>112</x:v>
@@ -44674,8 +44674,8 @@
       <x:c r="CN155" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CO155" t="s">
-        <x:v>1</x:v>
+      <x:c r="CO155" s="6" t="s">
+        <x:v>112</x:v>
       </x:c>
       <x:c r="CP155" s="6" t="s">
         <x:v>112</x:v>
@@ -44970,8 +44970,8 @@
       <x:c r="CN156" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CO156" t="s">
-        <x:v>1</x:v>
+      <x:c r="CO156" s="6" t="s">
+        <x:v>112</x:v>
       </x:c>
       <x:c r="CP156" s="6" t="s">
         <x:v>112</x:v>
@@ -45266,8 +45266,8 @@
       <x:c r="CN157" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CO157" t="s">
-        <x:v>1</x:v>
+      <x:c r="CO157" s="6" t="s">
+        <x:v>112</x:v>
       </x:c>
       <x:c r="CP157" t="s">
         <x:v>1</x:v>
@@ -45562,8 +45562,8 @@
       <x:c r="CN158" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CO158" t="s">
-        <x:v>1</x:v>
+      <x:c r="CO158" s="6" t="s">
+        <x:v>112</x:v>
       </x:c>
       <x:c r="CP158" s="6" t="s">
         <x:v>112</x:v>
@@ -47042,8 +47042,8 @@
       <x:c r="CN163" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CO163" t="s">
-        <x:v>1</x:v>
+      <x:c r="CO163" s="6" t="s">
+        <x:v>112</x:v>
       </x:c>
       <x:c r="CP163" t="s">
         <x:v>1</x:v>
@@ -47634,8 +47634,8 @@
       <x:c r="CN165" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CO165" t="s">
-        <x:v>1</x:v>
+      <x:c r="CO165" s="6" t="s">
+        <x:v>112</x:v>
       </x:c>
       <x:c r="CP165" t="s">
         <x:v>1</x:v>
@@ -50306,8 +50306,8 @@
       <x:c r="CN175" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CO175" t="s">
-        <x:v>1</x:v>
+      <x:c r="CO175" s="6" t="s">
+        <x:v>112</x:v>
       </x:c>
       <x:c r="CP175" s="6" t="s">
         <x:v>112</x:v>
@@ -50602,8 +50602,8 @@
       <x:c r="CN176" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CO176" t="s">
-        <x:v>1</x:v>
+      <x:c r="CO176" s="6" t="s">
+        <x:v>112</x:v>
       </x:c>
       <x:c r="CP176" s="6" t="s">
         <x:v>112</x:v>
@@ -50898,8 +50898,8 @@
       <x:c r="CN177" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CO177" t="s">
-        <x:v>1</x:v>
+      <x:c r="CO177" s="6" t="s">
+        <x:v>112</x:v>
       </x:c>
       <x:c r="CP177" s="6" t="s">
         <x:v>112</x:v>
@@ -51786,8 +51786,8 @@
       <x:c r="CN180" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CO180" t="s">
-        <x:v>1</x:v>
+      <x:c r="CO180" s="6" t="s">
+        <x:v>112</x:v>
       </x:c>
       <x:c r="CP180" s="6" t="s">
         <x:v>112</x:v>
@@ -52674,8 +52674,8 @@
       <x:c r="CN183" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CO183" t="s">
-        <x:v>1</x:v>
+      <x:c r="CO183" s="6" t="s">
+        <x:v>112</x:v>
       </x:c>
       <x:c r="CP183" s="6" t="s">
         <x:v>112</x:v>
@@ -52970,8 +52970,8 @@
       <x:c r="CN184" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CO184" t="s">
-        <x:v>1</x:v>
+      <x:c r="CO184" s="6" t="s">
+        <x:v>112</x:v>
       </x:c>
       <x:c r="CP184" t="s">
         <x:v>1</x:v>
@@ -60098,8 +60098,8 @@
       <x:c r="CN211" s="6" t="s">
         <x:v>112</x:v>
       </x:c>
-      <x:c r="CO211" s="6" t="s">
-        <x:v>112</x:v>
+      <x:c r="CO211" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="CP211" t="s">
         <x:v>1</x:v>

</xml_diff>

<commit_message>
Update REAL engines (C++, Python, Rust): 2026.9.2.
</commit_message>
<xml_diff>
--- a/RegexFeatureMatrix.xlsx
+++ b/RegexFeatureMatrix.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="R1860a50d809f4942"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="Rd78a55beea8e485d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -79,7 +79,7 @@
   </x:si>
   <x:si>
     <x:t>Python
- 3.14.6 </x:t>
+ 3.14.7 </x:t>
   </x:si>
   <x:si>
     <x:t>D
@@ -135,7 +135,7 @@
   </x:si>
   <x:si>
     <x:t>REAL
- 2026.8.20 </x:t>
+ 2026.9.2 </x:t>
   </x:si>
   <x:si>
     <x:t>Regex</x:t>

</xml_diff>